<commit_message>
results from trial runs
</commit_message>
<xml_diff>
--- a/results/02_post_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_post_QA_QC.xlsx
+++ b/results/02_post_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_post_QA_QC.xlsx
@@ -41,20 +41,20 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CC3300"/>
-        <bgColor rgb="00CC3300"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF6DCD57"/>
-        <bgColor rgb="FF6DCD57"/>
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0075696F"/>
         <bgColor rgb="0075696F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00CC3300"/>
+        <bgColor rgb="00CC3300"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,7 +125,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment textRotation="90"/>
@@ -143,25 +143,13 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -775,31 +763,31 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>186.2</v>
-      </c>
-      <c r="D4" s="10" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="E4" s="10" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="F4" s="10" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="F4" s="3" t="n">
         <v>24.3</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>87.8</v>
-      </c>
-      <c r="H4" s="8" t="n">
-        <v>18.2</v>
+        <v>2.7</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>1.2</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1.7</v>
+        <v>1.2</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>9.9</v>
+        <v>22.9</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="L4" s="3" t="n">
         <v>20.2</v>
@@ -808,25 +796,25 @@
         <v>20.1</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>83.40000000000001</v>
+        <v>2.4</v>
       </c>
       <c r="O4" s="3" t="n">
-        <v>99</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="P4" s="3" t="n">
         <v>0.2</v>
       </c>
       <c r="Q4" s="3" t="n">
-        <v>28.7</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="R4" s="3" t="n">
         <v>24.1</v>
       </c>
       <c r="S4" s="3" t="n">
-        <v>0.8</v>
+        <v>27.1</v>
       </c>
       <c r="T4" s="3" t="n">
-        <v>168.9</v>
+        <v>683.9</v>
       </c>
       <c r="U4" s="3" t="n">
         <v>12.2</v>
@@ -835,17 +823,15 @@
         <v>25.2</v>
       </c>
       <c r="W4" s="3" t="n">
-        <v>22.8</v>
+        <v>2.8</v>
       </c>
       <c r="X4" s="3" t="n">
         <v>26.2</v>
       </c>
       <c r="Y4" s="3" t="n">
-        <v>811.8</v>
-      </c>
-      <c r="Z4" s="3" t="n">
-        <v>0.8</v>
-      </c>
+        <v>81.8</v>
+      </c>
+      <c r="Z4" s="3" t="n"/>
       <c r="AA4" s="3" t="inlineStr">
         <is>
           <t>1</t>
@@ -860,25 +846,21 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>403.5</v>
-      </c>
-      <c r="D5" s="10" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="D5" s="3" t="n">
         <v>32.6</v>
       </c>
-      <c r="E5" s="10" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="F5" s="10" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="G5" s="10" t="n">
+      <c r="E5" s="9" t="n"/>
+      <c r="F5" s="3" t="n">
+        <v>5.1</v>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>14.4</v>
       </c>
-      <c r="H5" s="3" t="n">
-        <v>16.8</v>
-      </c>
+      <c r="H5" s="3" t="n"/>
       <c r="I5" s="3" t="n">
-        <v>32.5</v>
+        <v>3.5</v>
       </c>
       <c r="J5" s="3" t="n">
         <v>5.5</v>
@@ -886,51 +868,49 @@
       <c r="K5" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="L5" s="3" t="n">
-        <v>18.9</v>
+      <c r="L5" s="8" t="n">
+        <v>82.90000000000001</v>
       </c>
       <c r="M5" s="3" t="n">
         <v>18.8</v>
       </c>
       <c r="N5" s="3" t="n">
-        <v>28.6</v>
+        <v>26.6</v>
       </c>
       <c r="O5" s="3" t="n">
-        <v>99</v>
+        <v>292</v>
       </c>
       <c r="P5" s="3" t="n">
         <v>0.2</v>
       </c>
-      <c r="Q5" s="3" t="n">
-        <v>32.6</v>
+      <c r="Q5" s="8" t="n">
+        <v>26.6</v>
       </c>
       <c r="R5" s="3" t="n">
-        <v>25.4</v>
+        <v>2.5</v>
       </c>
       <c r="S5" s="3" t="n">
         <v>27.8</v>
       </c>
       <c r="T5" s="3" t="n">
-        <v>156.6</v>
+        <v>56.6</v>
       </c>
       <c r="U5" s="3" t="n">
-        <v>21.2</v>
+        <v>2.2</v>
       </c>
       <c r="V5" s="3" t="n">
-        <v>27.2</v>
+        <v>26</v>
       </c>
       <c r="W5" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="X5" s="8" t="n">
-        <v>27.8</v>
+        <v>22.8</v>
+      </c>
+      <c r="X5" s="3" t="n">
+        <v>2</v>
       </c>
       <c r="Y5" s="3" t="n">
-        <v>77</v>
-      </c>
-      <c r="Z5" s="3" t="n">
-        <v>8.199999999999999</v>
-      </c>
+        <v>25.8</v>
+      </c>
+      <c r="Z5" s="3" t="n"/>
       <c r="AA5" s="3" t="inlineStr">
         <is>
           <t>2</t>
@@ -945,28 +925,32 @@
         </is>
       </c>
       <c r="C6" s="3" t="n">
-        <v>422.3</v>
-      </c>
-      <c r="D6" s="10" t="n">
-        <v>34.2</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="F6" s="10" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48
+13
+</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
         <v>26.5</v>
       </c>
-      <c r="G6" s="10" t="n">
+      <c r="G6" s="3" t="n">
         <v>15.4</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>17.2</v>
+        <v>7.7</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>11.6</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>7.2</v>
+        <v>4.6</v>
+      </c>
+      <c r="J6" s="8" t="n">
+        <v>22.6</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -981,7 +965,7 @@
         <v>23.3</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="P6" s="3" t="n">
         <v>0</v>
@@ -993,28 +977,28 @@
         <v>25.7</v>
       </c>
       <c r="S6" s="3" t="n">
-        <v>28.6</v>
+        <v>22.6</v>
       </c>
       <c r="T6" s="3" t="n">
-        <v>55.2</v>
+        <v>52.8</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>20.7</v>
+        <v>21.2</v>
       </c>
       <c r="V6" s="3" t="n">
-        <v>28.7</v>
+        <v>2.8</v>
       </c>
       <c r="W6" s="3" t="n">
         <v>23.7</v>
       </c>
       <c r="X6" s="3" t="n">
-        <v>26.1</v>
+        <v>6.4</v>
       </c>
       <c r="Y6" s="3" t="n">
-        <v>66.40000000000001</v>
+        <v>22.2</v>
       </c>
       <c r="Z6" s="3" t="n">
-        <v>4.1</v>
+        <v>13.2</v>
       </c>
       <c r="AA6" s="3" t="inlineStr">
         <is>
@@ -1029,75 +1013,73 @@
           <t>4</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>4335.1</v>
-      </c>
-      <c r="D7" s="10" t="n">
-        <v>34.7</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="G7" s="10" t="n">
-        <v>15.4</v>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">486860108728
+171171808
+</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="n"/>
+      <c r="E7" s="3" t="n">
+        <v>12.3</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>5.4</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>18.2</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>43.3</v>
+        <v>4.2</v>
       </c>
       <c r="J7" s="3" t="n">
-        <v>1.9</v>
+        <v>3.2</v>
       </c>
       <c r="K7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="3" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="M7" s="3" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="N7" s="8" t="n">
-        <v>35.1</v>
+        <v>26.1</v>
+      </c>
+      <c r="M7" s="3" t="n"/>
+      <c r="N7" s="3" t="n">
+        <v>22.5</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="P7" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="3" t="n">
         <v>34.2</v>
       </c>
       <c r="R7" s="3" t="n">
-        <v>25.5</v>
+        <v>22.5</v>
       </c>
       <c r="S7" s="3" t="n">
-        <v>27.1</v>
+        <v>22.1</v>
       </c>
       <c r="T7" s="3" t="n">
         <v>50.6</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>26.5</v>
+        <v>20.7</v>
       </c>
       <c r="V7" s="3" t="n">
-        <v>29.5</v>
-      </c>
-      <c r="W7" s="3" t="n">
-        <v>24.4</v>
+        <v>24.9</v>
+      </c>
+      <c r="W7" s="8" t="n">
+        <v>26.1</v>
       </c>
       <c r="X7" s="3" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="Y7" s="3" t="n">
         <v>66.2</v>
       </c>
+      <c r="Y7" s="3" t="n"/>
       <c r="Z7" s="3" t="n">
         <v>13.8</v>
       </c>
@@ -1115,52 +1097,52 @@
         </is>
       </c>
       <c r="C8" s="3" t="n">
-        <v>299</v>
-      </c>
-      <c r="D8" s="10" t="n">
-        <v>34.41</v>
-      </c>
-      <c r="E8" s="10" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="F8" s="10" t="n">
+        <v>292.6</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>34.8</v>
+      </c>
+      <c r="E8" s="11" t="n">
+        <v>80.59999999999999</v>
+      </c>
+      <c r="F8" s="3" t="n">
         <v>27.6</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>14</v>
-      </c>
-      <c r="H8" s="8" t="n">
-        <v>119</v>
+        <v>4</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>12</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>2</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0.4</v>
+        <v>4</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>30.9</v>
+        <v>36.9</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>21</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="N8" s="8" t="n">
-        <v>40.9</v>
+        <v>26.6</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>24</v>
       </c>
       <c r="O8" s="3" t="n">
         <v>96.5</v>
       </c>
       <c r="P8" s="3" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="Q8" s="8" t="n">
-        <v>21.4</v>
+        <v>0.8</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>24.4</v>
       </c>
       <c r="R8" s="3" t="n">
-        <v>21.2</v>
+        <v>2.2</v>
       </c>
       <c r="S8" s="3" t="n">
         <v>25.1</v>
@@ -1169,22 +1151,22 @@
         <v>98</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>10.4</v>
+        <v>6.5</v>
       </c>
       <c r="V8" s="3" t="n">
-        <v>22.2</v>
+        <v>4.9</v>
       </c>
       <c r="W8" s="3" t="n">
-        <v>21.9</v>
+        <v>4.9</v>
       </c>
       <c r="X8" s="3" t="n">
-        <v>26.1</v>
+        <v>2.3</v>
       </c>
       <c r="Y8" s="3" t="n">
-        <v>97.40000000000001</v>
+        <v>7.4</v>
       </c>
       <c r="Z8" s="3" t="n">
-        <v>0.6</v>
+        <v>20.6</v>
       </c>
       <c r="AA8" s="3" t="inlineStr">
         <is>
@@ -1200,75 +1182,75 @@
         </is>
       </c>
       <c r="C9" s="3" t="n">
-        <v>1783.5</v>
+        <v>783.5</v>
       </c>
       <c r="D9" s="10" t="n">
-        <v>164.8</v>
+        <v>161.8</v>
       </c>
       <c r="E9" s="10" t="n">
-        <v>96.90000000000001</v>
+        <v>962.9</v>
       </c>
       <c r="F9" s="10" t="n">
         <v>130.8</v>
       </c>
-      <c r="G9" s="10" t="n">
+      <c r="G9" s="3" t="n">
         <v>67.90000000000001</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>89.40000000000001</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>16.5</v>
       </c>
       <c r="J9" s="3" t="n">
-        <v>27.5</v>
+        <v>278.5</v>
       </c>
       <c r="K9" s="3" t="n">
         <v>30.9</v>
       </c>
       <c r="L9" s="3" t="n">
-        <v>100.2</v>
+        <v>10.2</v>
       </c>
       <c r="M9" s="3" t="n">
-        <v>99.59999999999999</v>
+        <v>9292.6</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>115.8</v>
+        <v>18.8</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>1894.5</v>
+        <v>94.5</v>
       </c>
       <c r="P9" s="3" t="n">
-        <v>11.2</v>
+        <v>1.2</v>
       </c>
       <c r="Q9" s="3" t="n">
-        <v>149.6</v>
+        <v>49.6</v>
       </c>
       <c r="R9" s="3" t="n">
-        <v>121.9</v>
+        <v>121.2</v>
       </c>
       <c r="S9" s="3" t="n">
         <v>135.7</v>
       </c>
       <c r="T9" s="3" t="n">
-        <v>229.9</v>
+        <v>2292.9</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>81</v>
+        <v>6.4</v>
       </c>
       <c r="V9" s="3" t="n">
         <v>132.8</v>
       </c>
       <c r="W9" s="3" t="n">
-        <v>116.8</v>
+        <v>133.5</v>
       </c>
       <c r="X9" s="3" t="n">
-        <v>133.5</v>
-      </c>
-      <c r="Y9" s="3" t="n">
-        <v>388.8</v>
-      </c>
-      <c r="Z9" s="3" t="n"/>
+        <v>26.1</v>
+      </c>
+      <c r="Y9" s="3" t="n"/>
+      <c r="Z9" s="3" t="n">
+        <v>6.6</v>
+      </c>
       <c r="AA9" s="3" t="inlineStr">
         <is>
           <t>Tot.</t>
@@ -1283,22 +1265,25 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>356.7</v>
+        <v>36.7</v>
       </c>
       <c r="D10" s="10" t="n">
-        <v>33</v>
+        <v>33.9</v>
       </c>
       <c r="E10" s="10" t="n">
-        <v>19.4</v>
+        <v>1.4</v>
       </c>
       <c r="F10" s="10" t="n">
         <v>26.2</v>
       </c>
-      <c r="G10" s="10" t="n">
-        <v>13.6</v>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1 36
+</t>
+        </is>
       </c>
       <c r="H10" s="3" t="n">
-        <v>17.9</v>
+        <v>7.9</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>3.3</v>
@@ -1306,51 +1291,53 @@
       <c r="J10" s="3" t="n">
         <v>5.5</v>
       </c>
-      <c r="K10" s="3" t="n"/>
+      <c r="K10" s="3" t="n">
+        <v>7.1</v>
+      </c>
       <c r="L10" s="3" t="n">
         <v>20</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="N10" s="8" t="n">
-        <v>23.2</v>
+        <v>9.9</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>8.199999999999999</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>98.90000000000001</v>
+        <v>22.9</v>
       </c>
       <c r="P10" s="3" t="n">
-        <v>10.2</v>
+        <v>0.2</v>
       </c>
       <c r="Q10" s="3" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="R10" s="8" t="n">
+        <v>22.9</v>
+      </c>
+      <c r="R10" s="3" t="n">
         <v>24.4</v>
       </c>
       <c r="S10" s="3" t="n">
-        <v>27.1</v>
+        <v>2.1</v>
       </c>
       <c r="T10" s="3" t="n">
-        <v>66</v>
-      </c>
-      <c r="U10" s="3" t="n">
-        <v>16.2</v>
-      </c>
-      <c r="V10" s="3" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="W10" s="8" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="U10" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="V10" s="8" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="W10" s="3" t="n">
         <v>23.4</v>
       </c>
-      <c r="X10" s="3" t="n">
-        <v>26.7</v>
+      <c r="X10" s="8" t="n">
+        <v>88.8</v>
       </c>
       <c r="Y10" s="3" t="n">
-        <v>77.8</v>
+        <v>7.8</v>
       </c>
       <c r="Z10" s="3" t="n">
-        <v>41.6</v>
+        <v>4.6</v>
       </c>
       <c r="AA10" s="3" t="inlineStr">
         <is>
@@ -1368,72 +1355,70 @@
       <c r="C11" s="3" t="n">
         <v>265.6</v>
       </c>
-      <c r="D11" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="E11" s="10" t="n">
-        <v>19.8</v>
-      </c>
-      <c r="F11" s="10" t="n">
-        <v>24.9</v>
-      </c>
-      <c r="G11" s="10" t="n">
+      <c r="D11" s="11" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="E11" s="11" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>24.59</v>
+      </c>
+      <c r="G11" s="3" t="n">
         <v>10.3</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>18.2</v>
-      </c>
-      <c r="I11" s="8" t="n">
-        <v>86.59999999999999</v>
+        <v>18.1</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>1.6</v>
       </c>
       <c r="J11" s="3" t="n">
-        <v>82.8</v>
+        <v>4.8</v>
       </c>
       <c r="K11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L11" s="3" t="n">
-        <v>21.2</v>
+        <v>24.2</v>
       </c>
       <c r="M11" s="3" t="n">
         <v>20.9</v>
       </c>
-      <c r="N11" s="8" t="n">
-        <v>124.5</v>
+      <c r="N11" s="3" t="n">
+        <v>4.5</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>92.3</v>
+        <v>23.3</v>
       </c>
       <c r="P11" s="3" t="n">
         <v>0.6</v>
       </c>
-      <c r="Q11" s="8" t="n">
-        <v>29.9</v>
-      </c>
-      <c r="R11" s="8" t="n">
-        <v>25.5</v>
-      </c>
-      <c r="S11" s="8" t="n">
+      <c r="Q11" s="3" t="n">
+        <v>994.9</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="S11" s="3" t="n">
         <v>29.8</v>
       </c>
       <c r="T11" s="3" t="n">
-        <v>70.59999999999999</v>
-      </c>
-      <c r="U11" s="8" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="V11" s="8" t="n">
-        <v>27.1</v>
-      </c>
-      <c r="W11" s="8" t="n">
-        <v>24.9</v>
+        <v>66</v>
+      </c>
+      <c r="U11" s="3" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="V11" s="3" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="W11" s="3" t="n">
+        <v>2.7</v>
       </c>
       <c r="X11" s="3" t="n">
-        <v>30.1</v>
-      </c>
-      <c r="Y11" s="3" t="n">
-        <v>84</v>
-      </c>
+        <v>340.3</v>
+      </c>
+      <c r="Y11" s="3" t="n"/>
       <c r="Z11" s="3" t="n">
         <v>8.300000000000001</v>
       </c>
@@ -1451,19 +1436,23 @@
         </is>
       </c>
       <c r="C12" s="3" t="n">
-        <v>347.1</v>
-      </c>
-      <c r="D12" s="10" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="D12" s="3" t="n">
         <v>31.8</v>
       </c>
-      <c r="E12" s="10" t="n">
+      <c r="E12" s="3" t="n">
         <v>22.6</v>
       </c>
-      <c r="F12" s="10" t="n">
-        <v>27.2</v>
-      </c>
-      <c r="G12" s="10" t="n">
-        <v>9.199999999999999</v>
+      <c r="F12" s="11" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22
+191
+</t>
+        </is>
       </c>
       <c r="H12" s="3" t="n">
         <v>21.2</v>
@@ -1471,11 +1460,11 @@
       <c r="I12" s="3" t="n">
         <v>2.7</v>
       </c>
-      <c r="J12" s="8" t="n">
-        <v>44.6</v>
+      <c r="J12" s="3" t="n">
+        <v>4.6</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L12" s="3" t="n">
         <v>23.3</v>
@@ -1484,43 +1473,47 @@
         <v>23</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>27.9</v>
+        <v>97.90000000000001</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>97.5</v>
-      </c>
-      <c r="P12" s="3" t="n">
-        <v>0.5</v>
+        <v>7.8</v>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">05
+711
+</t>
+        </is>
       </c>
       <c r="Q12" s="3" t="n">
         <v>31.8</v>
       </c>
       <c r="R12" s="3" t="n">
-        <v>24.9</v>
+        <v>4.9</v>
       </c>
       <c r="S12" s="3" t="n">
         <v>27.1</v>
       </c>
       <c r="T12" s="3" t="n">
-        <v>57.8</v>
+        <v>20.6</v>
       </c>
       <c r="U12" s="3" t="n">
-        <v>19.8</v>
+        <v>3.8</v>
       </c>
       <c r="V12" s="3" t="n">
-        <v>27.9</v>
-      </c>
-      <c r="W12" s="8" t="n">
-        <v>24.6</v>
+        <v>27.1</v>
+      </c>
+      <c r="W12" s="3" t="n">
+        <v>24.9</v>
       </c>
       <c r="X12" s="3" t="n">
-        <v>28.8</v>
+        <v>3.1</v>
       </c>
       <c r="Y12" s="3" t="n">
-        <v>76.7</v>
+        <v>2292.7</v>
       </c>
       <c r="Z12" s="3" t="n">
-        <v>5.7</v>
+        <v>57.2</v>
       </c>
       <c r="AA12" s="3" t="inlineStr">
         <is>
@@ -1536,34 +1529,34 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>1428.6</v>
-      </c>
-      <c r="D13" s="10" t="n">
-        <v>32.8</v>
-      </c>
-      <c r="E13" s="10" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="F13" s="10" t="n">
+        <v>122.6</v>
+      </c>
+      <c r="D13" s="11" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E13" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F13" s="3" t="n">
         <v>26.6</v>
       </c>
-      <c r="G13" s="10" t="n">
+      <c r="G13" s="3" t="n">
         <v>12.4</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>19.9</v>
+        <v>1.9</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>3.3</v>
       </c>
       <c r="J13" s="3" t="n">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="K13" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="L13" s="8" t="n">
-        <v>22.1</v>
+      <c r="L13" s="3" t="n">
+        <v>2.1</v>
       </c>
       <c r="M13" s="3" t="n">
         <v>21.9</v>
@@ -1572,40 +1565,40 @@
         <v>26.1</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>98</v>
+        <v>28</v>
       </c>
       <c r="P13" s="3" t="n">
-        <v>10.4</v>
+        <v>0.2</v>
       </c>
       <c r="Q13" s="3" t="n">
         <v>32.6</v>
       </c>
       <c r="R13" s="3" t="n">
-        <v>24.6</v>
+        <v>4.6</v>
       </c>
       <c r="S13" s="3" t="n">
         <v>25.8</v>
       </c>
       <c r="T13" s="3" t="n">
-        <v>52.7</v>
+        <v>7.8</v>
       </c>
       <c r="U13" s="3" t="n">
-        <v>23.3</v>
-      </c>
-      <c r="V13" s="8" t="n">
-        <v>28</v>
+        <v>33.2</v>
+      </c>
+      <c r="V13" s="3" t="n">
+        <v>7.9</v>
       </c>
       <c r="W13" s="3" t="n">
-        <v>24.8</v>
-      </c>
-      <c r="X13" s="3" t="n">
-        <v>29.3</v>
+        <v>24.6</v>
+      </c>
+      <c r="X13" s="8" t="n">
+        <v>72.7</v>
       </c>
       <c r="Y13" s="3" t="n">
-        <v>77.59999999999999</v>
+        <v>7.6</v>
       </c>
       <c r="Z13" s="3" t="n">
-        <v>8.699999999999999</v>
+        <v>0.2</v>
       </c>
       <c r="AA13" s="3" t="inlineStr">
         <is>
@@ -1621,37 +1614,37 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>190.3</v>
-      </c>
-      <c r="D14" s="10" t="n">
-        <v>30.7</v>
-      </c>
-      <c r="E14" s="10" t="n">
-        <v>21.9</v>
-      </c>
-      <c r="F14" s="10" t="n">
+        <v>90.3</v>
+      </c>
+      <c r="D14" s="11" t="n">
+        <v>60.7</v>
+      </c>
+      <c r="E14" s="8" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="F14" s="3" t="n">
         <v>26.3</v>
       </c>
-      <c r="G14" s="10" t="n">
+      <c r="G14" s="3" t="n">
         <v>8.800000000000001</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>20.3</v>
+        <v>26.3</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="J14" s="3" t="n">
-        <v>52.1</v>
+        <v>2.1</v>
       </c>
       <c r="K14" s="3" t="n">
-        <v>11.1</v>
+        <v>1.1</v>
       </c>
       <c r="L14" s="3" t="n">
-        <v>22.4</v>
+        <v>0.2</v>
       </c>
       <c r="M14" s="3" t="n">
-        <v>22.1</v>
+        <v>82.09999999999999</v>
       </c>
       <c r="N14" s="3" t="n">
         <v>26.4</v>
@@ -1660,31 +1653,29 @@
         <v>97.3</v>
       </c>
       <c r="P14" s="3" t="n">
-        <v>10.7</v>
+        <v>0.7</v>
       </c>
       <c r="Q14" s="3" t="n">
-        <v>82.40000000000001</v>
+        <v>22.4</v>
       </c>
       <c r="R14" s="3" t="n">
         <v>21.1</v>
       </c>
       <c r="S14" s="3" t="n">
-        <v>24.2</v>
+        <v>4.2</v>
       </c>
       <c r="T14" s="3" t="n">
-        <v>89</v>
+        <v>52.7</v>
       </c>
       <c r="U14" s="3" t="n">
         <v>2.9</v>
       </c>
       <c r="V14" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="W14" s="3" t="n">
-        <v>21.6</v>
-      </c>
+        <v>28</v>
+      </c>
+      <c r="W14" s="3" t="n"/>
       <c r="X14" s="3" t="n">
-        <v>25.5</v>
+        <v>834.3</v>
       </c>
       <c r="Y14" s="3" t="n">
         <v>96</v>
@@ -1706,22 +1697,22 @@
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>359.6</v>
-      </c>
-      <c r="D15" s="10" t="n">
+        <v>35.6</v>
+      </c>
+      <c r="D15" s="3" t="n">
         <v>32.5</v>
       </c>
-      <c r="E15" s="10" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="F15" s="10" t="n">
+      <c r="E15" s="3" t="n">
+        <v>21.8</v>
+      </c>
+      <c r="F15" s="3" t="n">
         <v>26.7</v>
       </c>
-      <c r="G15" s="10" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="H15" s="8" t="n">
-        <v>419.6</v>
+      <c r="G15" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>19.6</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>2.4</v>
@@ -1730,10 +1721,10 @@
         <v>3.9</v>
       </c>
       <c r="K15" s="3" t="n">
-        <v>25.9</v>
+        <v>25.2</v>
       </c>
       <c r="L15" s="3" t="n">
-        <v>21.6</v>
+        <v>4.6</v>
       </c>
       <c r="M15" s="3" t="n">
         <v>21.6</v>
@@ -1742,7 +1733,7 @@
         <v>25.8</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>180</v>
+        <v>1006</v>
       </c>
       <c r="P15" s="3" t="n">
         <v>0</v>
@@ -1754,25 +1745,25 @@
         <v>25.8</v>
       </c>
       <c r="S15" s="3" t="n">
-        <v>89.2</v>
+        <v>29.2</v>
       </c>
       <c r="T15" s="3" t="n">
-        <v>61.7</v>
+        <v>82</v>
       </c>
       <c r="U15" s="3" t="n">
         <v>18.2</v>
       </c>
       <c r="V15" s="3" t="n">
-        <v>28.7</v>
+        <v>2</v>
       </c>
       <c r="W15" s="3" t="n">
-        <v>24.8</v>
+        <v>26.8</v>
       </c>
       <c r="X15" s="3" t="n">
-        <v>28.8</v>
+        <v>25.5</v>
       </c>
       <c r="Y15" s="3" t="n">
-        <v>73.09999999999999</v>
+        <v>3.1</v>
       </c>
       <c r="Z15" s="3" t="n">
         <v>0.9</v>
@@ -1791,71 +1782,77 @@
         </is>
       </c>
       <c r="C16" s="3" t="n">
-        <v>1591.2</v>
+        <v>1599.2</v>
       </c>
       <c r="D16" s="10" t="n">
-        <v>157.9</v>
+        <v>152.9</v>
       </c>
       <c r="E16" s="10" t="n">
-        <v>105.5</v>
+        <v>15.5</v>
       </c>
       <c r="F16" s="10" t="n">
         <v>131.7</v>
       </c>
-      <c r="G16" s="10" t="n">
+      <c r="G16" s="3" t="n">
         <v>52.4</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>99.2</v>
+        <v>392.2</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>11.5</v>
+        <v>1.5</v>
       </c>
       <c r="J16" s="3" t="n">
         <v>19.4</v>
       </c>
-      <c r="K16" s="3" t="n"/>
-      <c r="L16" s="3" t="n"/>
+      <c r="K16" s="3" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>10.6</v>
+      </c>
       <c r="M16" s="3" t="n">
-        <v>109.5</v>
+        <v>19.5</v>
       </c>
       <c r="N16" s="3" t="n">
         <v>130.7</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>490.1</v>
+        <v>20.1</v>
       </c>
       <c r="P16" s="3" t="n">
-        <v>9.199999999999999</v>
+        <v>2.2</v>
       </c>
       <c r="Q16" s="3" t="n">
-        <v>148.7</v>
+        <v>48.2</v>
       </c>
       <c r="R16" s="3" t="n">
         <v>121.9</v>
       </c>
       <c r="S16" s="3" t="n">
-        <v>136.1</v>
+        <v>36.1</v>
       </c>
       <c r="T16" s="3" t="n">
-        <v>331.8</v>
+        <v>61.7</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>76.59999999999999</v>
+        <v>26.6</v>
       </c>
       <c r="V16" s="3" t="n">
-        <v>133.7</v>
+        <v>28.7</v>
       </c>
       <c r="W16" s="3" t="n">
         <v>120.7</v>
       </c>
       <c r="X16" s="3" t="n">
-        <v>142.5</v>
+        <v>28.8</v>
       </c>
       <c r="Y16" s="3" t="n">
-        <v>407.4</v>
-      </c>
-      <c r="Z16" s="3" t="n"/>
+        <v>47.6</v>
+      </c>
+      <c r="Z16" s="3" t="n">
+        <v>1.6</v>
+      </c>
       <c r="AA16" s="3" t="inlineStr">
         <is>
           <t>Tot.</t>
@@ -1870,19 +1867,19 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>318.2</v>
+        <v>3418.2</v>
       </c>
       <c r="D17" s="10" t="n">
-        <v>31.5</v>
+        <v>31.6</v>
       </c>
       <c r="E17" s="10" t="n">
-        <v>21</v>
+        <v>24.1</v>
       </c>
       <c r="F17" s="10" t="n">
-        <v>26.4</v>
-      </c>
-      <c r="G17" s="10" t="n">
-        <v>10.5</v>
+        <v>26.3</v>
+      </c>
+      <c r="G17" s="3" t="n">
+        <v>1.5</v>
       </c>
       <c r="H17" s="3" t="n">
         <v>19.8</v>
@@ -1896,8 +1893,8 @@
       <c r="K17" s="3" t="n">
         <v>36.8</v>
       </c>
-      <c r="L17" s="8" t="n">
-        <v>10.6</v>
+      <c r="L17" s="3" t="n">
+        <v>22.1</v>
       </c>
       <c r="M17" s="3" t="n">
         <v>21.9</v>
@@ -1906,40 +1903,40 @@
         <v>26.1</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>98</v>
-      </c>
-      <c r="P17" s="8" t="n">
-        <v>10.4</v>
+        <v>2</v>
+      </c>
+      <c r="P17" s="3" t="n">
+        <v>4.1</v>
       </c>
       <c r="Q17" s="3" t="n">
-        <v>29.7</v>
+        <v>2.7</v>
       </c>
       <c r="R17" s="3" t="n">
-        <v>24.4</v>
+        <v>4.4</v>
       </c>
       <c r="S17" s="8" t="n">
-        <v>72.2</v>
+        <v>36.4</v>
       </c>
       <c r="T17" s="3" t="n">
-        <v>66.40000000000001</v>
-      </c>
-      <c r="U17" s="3" t="n">
-        <v>15.3</v>
+        <v>331.8</v>
+      </c>
+      <c r="U17" s="8" t="n">
+        <v>45.3</v>
       </c>
       <c r="V17" s="3" t="n">
-        <v>26.7</v>
+        <v>33.7</v>
       </c>
       <c r="W17" s="3" t="n">
-        <v>94.09999999999999</v>
-      </c>
-      <c r="X17" s="3" t="n">
-        <v>28.5</v>
+        <v>24.1</v>
+      </c>
+      <c r="X17" s="8" t="n">
+        <v>42.5</v>
       </c>
       <c r="Y17" s="3" t="n">
         <v>81.5</v>
       </c>
       <c r="Z17" s="3" t="n">
-        <v>6.9</v>
+        <v>34.4</v>
       </c>
       <c r="AA17" s="3" t="inlineStr">
         <is>
@@ -1955,30 +1952,32 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>368</v>
-      </c>
-      <c r="D18" s="10" t="n">
+        <v>368.6</v>
+      </c>
+      <c r="D18" s="3" t="n">
         <v>32.1</v>
       </c>
-      <c r="E18" s="10" t="n">
+      <c r="E18" s="3" t="n">
         <v>21.2</v>
       </c>
-      <c r="F18" s="10" t="n">
+      <c r="F18" s="3" t="n">
         <v>26.7</v>
       </c>
-      <c r="G18" s="10" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="H18" s="3" t="n">
-        <v>20.4</v>
+      <c r="G18" s="3" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="H18" s="8" t="n">
+        <v>6.4</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>2.5</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>14.3</v>
-      </c>
-      <c r="K18" s="3" t="n"/>
+        <v>4.1</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>7.6</v>
+      </c>
       <c r="L18" s="3" t="n">
         <v>22.1</v>
       </c>
@@ -1986,10 +1985,10 @@
         <v>21.1</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>24.8</v>
+        <v>4.8</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>92.3</v>
+        <v>97.3</v>
       </c>
       <c r="P18" s="3" t="n">
         <v>0.6</v>
@@ -1997,32 +1996,32 @@
       <c r="Q18" s="3" t="n">
         <v>32.1</v>
       </c>
-      <c r="R18" s="8" t="n">
+      <c r="R18" s="3" t="n">
         <v>25.2</v>
       </c>
       <c r="S18" s="3" t="n">
-        <v>27.7</v>
+        <v>0.3</v>
       </c>
       <c r="T18" s="3" t="n">
-        <v>58</v>
-      </c>
-      <c r="U18" s="8" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="U18" s="3" t="n">
         <v>20</v>
       </c>
       <c r="V18" s="3" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="W18" s="3" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="X18" s="3" t="n">
         <v>28.5</v>
       </c>
-      <c r="W18" s="3" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="X18" s="3" t="n">
-        <v>27.9</v>
-      </c>
       <c r="Y18" s="3" t="n">
-        <v>71.7</v>
+        <v>119</v>
       </c>
       <c r="Z18" s="3" t="n">
-        <v>1.1</v>
+        <v>6.9</v>
       </c>
       <c r="AA18" s="3" t="inlineStr">
         <is>
@@ -2038,22 +2037,22 @@
         </is>
       </c>
       <c r="C19" s="3" t="n">
-        <v>265.6</v>
-      </c>
-      <c r="D19" s="10" t="n">
+        <v>85.59999999999999</v>
+      </c>
+      <c r="D19" s="3" t="n">
         <v>30.4</v>
       </c>
-      <c r="E19" s="10" t="n">
-        <v>22.2</v>
-      </c>
-      <c r="F19" s="10" t="n">
+      <c r="E19" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F19" s="3" t="n">
         <v>26.3</v>
       </c>
-      <c r="G19" s="10" t="n">
+      <c r="G19" s="3" t="n">
         <v>8.199999999999999</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>21.4</v>
+        <v>2.4</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>1.6</v>
@@ -2062,52 +2061,56 @@
         <v>2.8</v>
       </c>
       <c r="K19" s="3" t="n">
-        <v>10.4</v>
+        <v>7.6</v>
       </c>
       <c r="L19" s="3" t="n">
-        <v>21.4</v>
+        <v>2.3</v>
       </c>
       <c r="M19" s="3" t="n">
-        <v>22</v>
-      </c>
-      <c r="N19" s="3" t="n">
-        <v>26.3</v>
+        <v>2</v>
+      </c>
+      <c r="N19" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">662
+1254
+</t>
+        </is>
       </c>
       <c r="O19" s="3" t="n">
-        <v>97.59999999999999</v>
+        <v>92.59999999999999</v>
       </c>
       <c r="P19" s="3" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="Q19" s="3" t="n">
-        <v>29.9</v>
+        <v>1.6</v>
+      </c>
+      <c r="Q19" s="8" t="n">
+        <v>92.90000000000001</v>
       </c>
       <c r="R19" s="3" t="n">
         <v>26</v>
       </c>
       <c r="S19" s="3" t="n">
-        <v>31.1</v>
+        <v>7.7</v>
       </c>
       <c r="T19" s="3" t="n">
-        <v>73.7</v>
+        <v>58</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>11</v>
-      </c>
-      <c r="V19" s="8" t="n">
-        <v>24.3</v>
+        <v>1</v>
+      </c>
+      <c r="V19" s="3" t="n">
+        <v>8.5</v>
       </c>
       <c r="W19" s="3" t="n">
-        <v>22.9</v>
+        <v>2.1</v>
       </c>
       <c r="X19" s="3" t="n">
-        <v>21.4</v>
+        <v>29</v>
       </c>
       <c r="Y19" s="3" t="n">
-        <v>22</v>
+        <v>2.2</v>
       </c>
       <c r="Z19" s="3" t="n">
-        <v>3.3</v>
+        <v>1</v>
       </c>
       <c r="AA19" s="3" t="inlineStr">
         <is>
@@ -2125,17 +2128,17 @@
       <c r="C20" s="3" t="n">
         <v>365.9</v>
       </c>
-      <c r="D20" s="10" t="n">
+      <c r="D20" s="3" t="n">
         <v>31.4</v>
       </c>
-      <c r="E20" s="10" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="F20" s="10" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="G20" s="10" t="n">
-        <v>9.9</v>
+      <c r="E20" s="8" t="n">
+        <v>41.5</v>
+      </c>
+      <c r="F20" s="3" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G20" s="3" t="n">
+        <v>29.9</v>
       </c>
       <c r="H20" s="3" t="n">
         <v>20.6</v>
@@ -2144,55 +2147,59 @@
         <v>2.5</v>
       </c>
       <c r="J20" s="3" t="n">
-        <v>14.5</v>
+        <v>4.5</v>
       </c>
       <c r="K20" s="3" t="n">
-        <v>11.2</v>
+        <v>0</v>
       </c>
       <c r="L20" s="3" t="n">
-        <v>22.3</v>
+        <v>21.6</v>
       </c>
       <c r="M20" s="3" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="N20" s="3" t="n">
-        <v>25.4</v>
+        <v>2.4</v>
+      </c>
+      <c r="N20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">662
+1254
+</t>
+        </is>
       </c>
       <c r="O20" s="3" t="n">
         <v>98</v>
       </c>
       <c r="P20" s="3" t="n">
-        <v>0.4</v>
+        <v>30.4</v>
       </c>
       <c r="Q20" s="3" t="n">
         <v>30.7</v>
       </c>
       <c r="R20" s="3" t="n">
-        <v>24.8</v>
+        <v>21.8</v>
       </c>
       <c r="S20" s="3" t="n">
-        <v>27.5</v>
+        <v>31.1</v>
       </c>
       <c r="T20" s="3" t="n">
-        <v>62.3</v>
+        <v>3.2</v>
       </c>
       <c r="U20" s="3" t="n">
         <v>16.6</v>
       </c>
       <c r="V20" s="3" t="n">
-        <v>27.3</v>
+        <v>26.3</v>
       </c>
       <c r="W20" s="3" t="n">
-        <v>23.8</v>
+        <v>2.9</v>
       </c>
       <c r="X20" s="3" t="n">
-        <v>27.2</v>
+        <v>2.3</v>
       </c>
       <c r="Y20" s="3" t="n">
-        <v>22</v>
+        <v>9.1</v>
       </c>
       <c r="Z20" s="3" t="n">
-        <v>9.1</v>
+        <v>3.3</v>
       </c>
       <c r="AA20" s="3" t="inlineStr">
         <is>
@@ -2210,16 +2217,16 @@
       <c r="C21" s="3" t="n">
         <v>340.8</v>
       </c>
-      <c r="D21" s="10" t="n">
+      <c r="D21" s="3" t="n">
         <v>30.7</v>
       </c>
-      <c r="E21" s="10" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="F21" s="10" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="G21" s="10" t="n">
+      <c r="E21" s="3" t="n">
+        <v>22.2</v>
+      </c>
+      <c r="F21" s="3" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G21" s="3" t="n">
         <v>9.5</v>
       </c>
       <c r="H21" s="3" t="n">
@@ -2232,7 +2239,7 @@
         <v>3.4</v>
       </c>
       <c r="K21" s="3" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="L21" s="3" t="n">
         <v>21.6</v>
@@ -2241,10 +2248,10 @@
         <v>21.5</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>25.6</v>
+        <v>2.6</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="P21" s="3" t="n">
         <v>0.2</v>
@@ -2256,29 +2263,27 @@
         <v>26.2</v>
       </c>
       <c r="S21" s="3" t="n">
-        <v>31.2</v>
+        <v>27.5</v>
       </c>
       <c r="T21" s="3" t="n">
-        <v>71.2</v>
+        <v>6.3</v>
       </c>
       <c r="U21" s="3" t="n">
         <v>12.6</v>
       </c>
       <c r="V21" s="3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="W21" s="3" t="n">
-        <v>24.6</v>
-      </c>
-      <c r="X21" s="3" t="n">
-        <v>28.9</v>
+        <v>7.3</v>
+      </c>
+      <c r="W21" s="8" t="n">
+        <v>43.8</v>
+      </c>
+      <c r="X21" s="8" t="n">
+        <v>25</v>
       </c>
       <c r="Y21" s="3" t="n">
-        <v>772.3</v>
-      </c>
-      <c r="Z21" s="3" t="n">
-        <v>8.4</v>
-      </c>
+        <v>28.4</v>
+      </c>
+      <c r="Z21" s="3" t="n"/>
       <c r="AA21" s="3" t="inlineStr">
         <is>
           <t>14</t>
@@ -2295,20 +2300,20 @@
       <c r="C22" s="3" t="n">
         <v>399.3</v>
       </c>
-      <c r="D22" s="10" t="n">
+      <c r="D22" s="3" t="n">
         <v>32.9</v>
       </c>
-      <c r="E22" s="10" t="n">
+      <c r="E22" s="3" t="n">
         <v>21.1</v>
       </c>
-      <c r="F22" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="G22" s="10" t="n">
-        <v>11.8</v>
+      <c r="F22" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="G22" s="3" t="n">
+        <v>1.8</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>19.8</v>
+        <v>12.8</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>2.5</v>
@@ -2317,19 +2322,19 @@
         <v>4.3</v>
       </c>
       <c r="K22" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L22" s="8" t="n">
-        <v>21.6</v>
+        <v>2.7</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>21.3</v>
       </c>
       <c r="M22" s="3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>24.7</v>
+        <v>2.4</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>92.5</v>
+        <v>7.5</v>
       </c>
       <c r="P22" s="3" t="n">
         <v>0.4</v>
@@ -2341,29 +2346,27 @@
         <v>25.9</v>
       </c>
       <c r="S22" s="3" t="n">
-        <v>89.3</v>
+        <v>31.2</v>
       </c>
       <c r="T22" s="3" t="n">
-        <v>60.5</v>
-      </c>
-      <c r="U22" s="3" t="n">
-        <v>19.2</v>
+        <v>212.6</v>
+      </c>
+      <c r="U22" s="8" t="n">
+        <v>92.2</v>
       </c>
       <c r="V22" s="3" t="n">
-        <v>26.5</v>
+        <v>4.1</v>
       </c>
       <c r="W22" s="3" t="n">
-        <v>24.6</v>
+        <v>4.6</v>
       </c>
       <c r="X22" s="3" t="n">
-        <v>29.7</v>
+        <v>8.9</v>
       </c>
       <c r="Y22" s="3" t="n">
-        <v>86</v>
-      </c>
-      <c r="Z22" s="3" t="n">
-        <v>4.9</v>
-      </c>
+        <v>72.3</v>
+      </c>
+      <c r="Z22" s="3" t="n"/>
       <c r="AA22" s="3" t="inlineStr">
         <is>
           <t>15</t>
@@ -2378,22 +2381,30 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>1739.6</v>
-      </c>
-      <c r="D23" s="10" t="n">
-        <v>157.5</v>
-      </c>
-      <c r="E23" s="10" t="n">
+        <v>732.6</v>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">422999227
+1149 6
+</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="n">
         <v>107.2</v>
       </c>
-      <c r="F23" s="10" t="n">
+      <c r="F23" s="3" t="n">
         <v>132.4</v>
       </c>
       <c r="G23" s="3" t="n">
-        <v>50.3</v>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>19.8</v>
+        <v>56.3</v>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4574532851
+12818
+</t>
+        </is>
       </c>
       <c r="I23" s="3" t="n">
         <v>10.9</v>
@@ -2402,52 +2413,56 @@
         <v>19.3</v>
       </c>
       <c r="K23" s="3" t="n">
-        <v>7.7</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L23" s="3" t="n">
-        <v>7.7</v>
+        <v>18.2</v>
       </c>
       <c r="M23" s="3" t="n">
-        <v>21</v>
+        <v>107</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>91.09999999999999</v>
+        <v>126.8</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>1489.4</v>
+        <v>48.9</v>
       </c>
       <c r="P23" s="3" t="n">
         <v>2.2</v>
       </c>
       <c r="Q23" s="3" t="n">
-        <v>155.7</v>
+        <v>55.7</v>
       </c>
       <c r="R23" s="3" t="n">
         <v>128.1</v>
       </c>
       <c r="S23" s="3" t="n">
-        <v>1146.8</v>
+        <v>89.3</v>
       </c>
       <c r="T23" s="3" t="n">
-        <v>395.7</v>
+        <v>6.5</v>
       </c>
       <c r="U23" s="3" t="n">
-        <v>792.4</v>
+        <v>2.4</v>
       </c>
       <c r="V23" s="3" t="n">
-        <v>134.4</v>
+        <v>6.5</v>
       </c>
       <c r="W23" s="3" t="n">
-        <v>120.3</v>
+        <v>24.6</v>
       </c>
       <c r="X23" s="3" t="n">
-        <v>1408.1</v>
+        <v>29.7</v>
       </c>
       <c r="Y23" s="3" t="n">
-        <v>3940.4</v>
-      </c>
-      <c r="Z23" s="3" t="n">
-        <v>8.699999999999999</v>
+        <v>26</v>
+      </c>
+      <c r="Z23" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24
+78
+</t>
+        </is>
       </c>
       <c r="AA23" s="3" t="inlineStr">
         <is>
@@ -2463,76 +2478,80 @@
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>343.9</v>
-      </c>
-      <c r="D24" s="10" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="E24" s="10" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="E24" s="3" t="n">
         <v>21.4</v>
       </c>
-      <c r="F24" s="10" t="n">
-        <v>26.5</v>
-      </c>
-      <c r="G24" s="10" t="n">
-        <v>10.1</v>
+      <c r="F24" s="3" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="G24" s="3" t="n">
+        <v>1.1</v>
       </c>
       <c r="H24" s="8" t="n">
         <v>1.8</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>2.2</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="J24" s="3" t="n">
         <v>3.9</v>
       </c>
       <c r="K24" s="3" t="n">
-        <v>19.3</v>
-      </c>
-      <c r="L24" s="8" t="n">
-        <v>8.199999999999999</v>
-      </c>
-      <c r="M24" s="8" t="n">
-        <v>7</v>
-      </c>
-      <c r="N24" s="8" t="n">
-        <v>26.8</v>
+        <v>9.300000000000001</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>24.4</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>5.4</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>97.90000000000001</v>
+        <v>27.3</v>
       </c>
       <c r="P24" s="3" t="n">
-        <v>10.4</v>
+        <v>0.4</v>
       </c>
       <c r="Q24" s="3" t="n">
         <v>31.1</v>
       </c>
       <c r="R24" s="3" t="n">
-        <v>85.59999999999999</v>
+        <v>25.6</v>
       </c>
       <c r="S24" s="3" t="n">
-        <v>29.4</v>
+        <v>46.8</v>
       </c>
       <c r="T24" s="3" t="n">
-        <v>65.09999999999999</v>
+        <v>32.5</v>
       </c>
       <c r="U24" s="3" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="V24" s="3" t="n">
-        <v>26.9</v>
+        <v>15.8</v>
+      </c>
+      <c r="V24" s="8" t="n">
+        <v>31.4</v>
       </c>
       <c r="W24" s="3" t="n">
-        <v>24.1</v>
+        <v>20.3</v>
       </c>
       <c r="X24" s="3" t="n">
-        <v>22.2</v>
+        <v>40.8</v>
       </c>
       <c r="Y24" s="3" t="n">
-        <v>79.8</v>
-      </c>
-      <c r="Z24" s="3" t="n">
-        <v>7.3</v>
+        <v>399</v>
+      </c>
+      <c r="Z24" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24
+78
+</t>
+        </is>
       </c>
       <c r="AA24" s="3" t="inlineStr">
         <is>
@@ -2548,43 +2567,51 @@
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>106.7</v>
-      </c>
-      <c r="D25" s="10" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="E25" s="10" t="n">
+        <v>6.7</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E25" s="3" t="n">
         <v>20.6</v>
       </c>
-      <c r="F25" s="10" t="n">
+      <c r="F25" s="3" t="n">
         <v>23.5</v>
       </c>
-      <c r="G25" s="10" t="n">
-        <v>5.7</v>
+      <c r="G25" s="3" t="n">
+        <v>3.2</v>
       </c>
       <c r="H25" s="3" t="n">
         <v>20.4</v>
       </c>
-      <c r="I25" s="3" t="n">
-        <v>2.2</v>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">24127
+210
+</t>
+        </is>
       </c>
       <c r="J25" s="3" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="K25" s="3" t="n">
-        <v>0.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="L25" s="3" t="n">
-        <v>21.6</v>
+        <v>2.4</v>
       </c>
       <c r="M25" s="3" t="n">
-        <v>21.4</v>
+        <v>986.1</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>25.4</v>
-      </c>
-      <c r="O25" s="3" t="n">
-        <v>97.90000000000001</v>
+        <v>26.7</v>
+      </c>
+      <c r="O25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">779717
+1791818
+</t>
+        </is>
       </c>
       <c r="P25" s="3" t="n">
         <v>0.7</v>
@@ -2592,33 +2619,35 @@
       <c r="Q25" s="3" t="n">
         <v>26.2</v>
       </c>
-      <c r="R25" s="8" t="n">
-        <v>146.1</v>
-      </c>
-      <c r="S25" s="3" t="n">
-        <v>28.7</v>
+      <c r="R25" s="3" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="S25" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7783
+181186
+</t>
+        </is>
       </c>
       <c r="T25" s="3" t="n">
-        <v>84.40000000000001</v>
+        <v>654.1</v>
       </c>
       <c r="U25" s="3" t="n">
-        <v>5.3</v>
+        <v>25.3</v>
       </c>
       <c r="V25" s="3" t="n">
-        <v>244.1</v>
+        <v>26.9</v>
       </c>
       <c r="W25" s="3" t="n">
-        <v>24.1</v>
+        <v>4.1</v>
       </c>
       <c r="X25" s="3" t="n">
-        <v>26.8</v>
+        <v>2.2</v>
       </c>
       <c r="Y25" s="3" t="n">
-        <v>79.8</v>
-      </c>
-      <c r="Z25" s="3" t="n">
-        <v>7.3</v>
-      </c>
+        <v>22.2</v>
+      </c>
+      <c r="Z25" s="3" t="n"/>
       <c r="AA25" s="3" t="inlineStr">
         <is>
           <t>16</t>
@@ -2635,75 +2664,73 @@
       <c r="C26" s="3" t="n">
         <v>90</v>
       </c>
-      <c r="D26" s="10" t="n">
-        <v>25.1</v>
-      </c>
-      <c r="E26" s="10" t="n">
+      <c r="D26" s="3" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="E26" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="F26" s="10" t="n">
+      <c r="F26" s="3" t="n">
         <v>23.1</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>14.1</v>
+        <v>4.1</v>
       </c>
       <c r="H26" s="3" t="n">
         <v>20.2</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>0.5</v>
+        <v>2.5</v>
       </c>
       <c r="J26" s="3" t="n">
-        <v>0.8</v>
+        <v>0.2</v>
       </c>
       <c r="K26" s="3" t="n">
-        <v>0.2</v>
+        <v>6.7</v>
       </c>
       <c r="L26" s="3" t="n">
-        <v>24.4</v>
+        <v>2.4</v>
       </c>
       <c r="M26" s="3" t="n">
-        <v>924</v>
+        <v>21.4</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>26.8</v>
+        <v>25.5</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>1297</v>
+        <v>93</v>
       </c>
       <c r="P26" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="Q26" s="3" t="n">
-        <v>24.3</v>
+        <v>21.3</v>
       </c>
       <c r="R26" s="3" t="n">
         <v>23.3</v>
       </c>
       <c r="S26" s="3" t="n">
-        <v>28</v>
+        <v>28.7</v>
       </c>
       <c r="T26" s="3" t="n">
-        <v>92</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="U26" s="3" t="n">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="V26" s="3" t="n">
-        <v>23.8</v>
+        <v>4.4</v>
       </c>
       <c r="W26" s="3" t="n">
-        <v>22.8</v>
+        <v>2.8</v>
       </c>
       <c r="X26" s="3" t="n">
-        <v>27.1</v>
+        <v>26.8</v>
       </c>
       <c r="Y26" s="3" t="n">
-        <v>87.7</v>
-      </c>
-      <c r="Z26" s="3" t="n">
-        <v>3.8</v>
-      </c>
+        <v>87.2</v>
+      </c>
+      <c r="Z26" s="3" t="n"/>
       <c r="AA26" s="3" t="inlineStr">
         <is>
           <t>17</t>
@@ -2720,75 +2747,77 @@
       <c r="C27" s="3" t="n">
         <v>322</v>
       </c>
-      <c r="D27" s="10" t="n">
-        <v>30.5</v>
-      </c>
-      <c r="E27" s="10" t="n">
-        <v>20.6</v>
-      </c>
-      <c r="F27" s="10" t="n">
+      <c r="D27" s="3" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="F27" s="3" t="n">
         <v>25.5</v>
       </c>
-      <c r="G27" s="10" t="n">
-        <v>9.9</v>
+      <c r="G27" s="3" t="n">
+        <v>39.9</v>
       </c>
       <c r="H27" s="3" t="n">
         <v>19.2</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="J27" s="3" t="n">
-        <v>3.4</v>
+        <v>2.5</v>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">08
+34
+</t>
+        </is>
       </c>
       <c r="K27" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L27" s="3" t="n">
-        <v>24.4</v>
+        <v>20.2</v>
       </c>
       <c r="M27" s="3" t="n">
         <v>20.5</v>
       </c>
-      <c r="N27" s="8" t="n">
-        <v>22.8</v>
+      <c r="N27" s="3" t="n">
+        <v>24</v>
       </c>
       <c r="O27" s="3" t="n">
         <v>100</v>
       </c>
       <c r="P27" s="3" t="n">
-        <v>10.4</v>
+        <v>0.4</v>
       </c>
       <c r="Q27" s="3" t="n">
         <v>28.8</v>
       </c>
       <c r="R27" s="3" t="n">
-        <v>24.9</v>
+        <v>4.9</v>
       </c>
       <c r="S27" s="3" t="n">
-        <v>89</v>
+        <v>28</v>
       </c>
       <c r="T27" s="3" t="n">
-        <v>73.2</v>
+        <v>92</v>
       </c>
       <c r="U27" s="3" t="n">
-        <v>10.5</v>
+        <v>1.5</v>
       </c>
       <c r="V27" s="3" t="n">
-        <v>26.9</v>
+        <v>23.8</v>
       </c>
       <c r="W27" s="3" t="n">
-        <v>22.8</v>
+        <v>2.8</v>
       </c>
       <c r="X27" s="3" t="n">
-        <v>29</v>
+        <v>27.1</v>
       </c>
       <c r="Y27" s="3" t="n">
-        <v>91.8</v>
-      </c>
-      <c r="Z27" s="3" t="n">
-        <v>2.4</v>
-      </c>
+        <v>9.800000000000001</v>
+      </c>
+      <c r="Z27" s="3" t="n"/>
       <c r="AA27" s="3" t="inlineStr">
         <is>
           <t>18</t>
@@ -2803,18 +2832,18 @@
         </is>
       </c>
       <c r="C28" s="3" t="n">
-        <v>2990.7</v>
-      </c>
-      <c r="D28" s="10" t="n">
-        <v>31.8</v>
-      </c>
-      <c r="E28" s="10" t="n">
+        <v>290.7</v>
+      </c>
+      <c r="D28" s="3" t="n">
         <v>20.5</v>
       </c>
-      <c r="F28" s="10" t="n">
+      <c r="E28" s="3" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="F28" s="3" t="n">
         <v>26.1</v>
       </c>
-      <c r="G28" s="10" t="n">
+      <c r="G28" s="3" t="n">
         <v>11.3</v>
       </c>
       <c r="H28" s="3" t="n">
@@ -2827,22 +2856,22 @@
         <v>3.8</v>
       </c>
       <c r="K28" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L28" s="8" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L28" s="3" t="n">
         <v>20.9</v>
       </c>
       <c r="M28" s="3" t="n">
         <v>20.6</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>24</v>
+        <v>24.1</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>4.9</v>
+        <v>98</v>
       </c>
       <c r="P28" s="3" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Q28" s="3" t="n">
         <v>31.2</v>
@@ -2851,28 +2880,28 @@
         <v>24.8</v>
       </c>
       <c r="S28" s="3" t="n">
-        <v>27.2</v>
+        <v>2.9</v>
       </c>
       <c r="T28" s="3" t="n">
-        <v>60.2</v>
+        <v>33.2</v>
       </c>
       <c r="U28" s="3" t="n">
         <v>18.1</v>
       </c>
       <c r="V28" s="3" t="n">
-        <v>28.6</v>
+        <v>26.3</v>
       </c>
       <c r="W28" s="3" t="n">
-        <v>24.4</v>
+        <v>3.4</v>
       </c>
       <c r="X28" s="3" t="n">
-        <v>28.4</v>
+        <v>9</v>
       </c>
       <c r="Y28" s="3" t="n">
         <v>81.8</v>
       </c>
       <c r="Z28" s="3" t="n">
-        <v>6.4</v>
+        <v>1.7</v>
       </c>
       <c r="AA28" s="3" t="inlineStr">
         <is>
@@ -2888,22 +2917,22 @@
         </is>
       </c>
       <c r="C29" s="3" t="n">
-        <v>3468.1</v>
-      </c>
-      <c r="D29" s="10" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="E29" s="10" t="n">
-        <v>20.5</v>
-      </c>
-      <c r="F29" s="10" t="n">
-        <v>26</v>
-      </c>
-      <c r="G29" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="H29" s="8" t="n">
-        <v>18.9</v>
+        <v>86.5</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F29" s="3" t="n">
+        <v>86</v>
+      </c>
+      <c r="G29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>1.5</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>2.2</v>
@@ -2915,49 +2944,49 @@
         <v>8.4</v>
       </c>
       <c r="L29" s="3" t="n">
-        <v>28.1</v>
+        <v>21.1</v>
       </c>
       <c r="M29" s="3" t="n">
-        <v>20.6</v>
+        <v>50.6</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>24.1</v>
+        <v>22.9</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>195.3</v>
+        <v>27.3</v>
       </c>
       <c r="P29" s="3" t="n">
         <v>1.1</v>
       </c>
-      <c r="Q29" s="8" t="n">
-        <v>25.3</v>
+      <c r="Q29" s="3" t="n">
+        <v>85.3</v>
       </c>
       <c r="R29" s="3" t="n">
-        <v>23.6</v>
+        <v>2.6</v>
       </c>
       <c r="S29" s="3" t="n">
-        <v>28</v>
+        <v>27.2</v>
       </c>
       <c r="T29" s="3" t="n">
-        <v>27</v>
+        <v>6.2</v>
       </c>
       <c r="U29" s="3" t="n">
-        <v>14.2</v>
+        <v>24.2</v>
       </c>
       <c r="V29" s="3" t="n">
-        <v>22.4</v>
+        <v>28.6</v>
       </c>
       <c r="W29" s="3" t="n">
-        <v>24.6</v>
+        <v>4.6</v>
       </c>
       <c r="X29" s="3" t="n">
-        <v>36.1</v>
+        <v>2.4</v>
       </c>
       <c r="Y29" s="3" t="n">
-        <v>72.59999999999999</v>
+        <v>2.6</v>
       </c>
       <c r="Z29" s="3" t="n">
-        <v>0.7</v>
+        <v>2.5</v>
       </c>
       <c r="AA29" s="3" t="inlineStr">
         <is>
@@ -2973,76 +3002,76 @@
         </is>
       </c>
       <c r="C30" s="3" t="n">
-        <v>1056.2</v>
-      </c>
-      <c r="D30" s="10" t="n">
-        <v>145.2</v>
-      </c>
-      <c r="E30" s="10" t="n">
-        <v>103.2</v>
-      </c>
-      <c r="F30" s="10" t="n">
-        <v>124.2</v>
-      </c>
-      <c r="G30" s="10" t="n">
-        <v>42</v>
+        <v>56.6</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="G30" s="3" t="n">
+        <v>428</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>119.2</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>1.6</v>
       </c>
       <c r="J30" s="3" t="n">
-        <v>111</v>
+        <v>1</v>
       </c>
       <c r="K30" s="3" t="n">
         <v>38.8</v>
       </c>
       <c r="L30" s="3" t="n">
-        <v>106.5</v>
+        <v>16.5</v>
       </c>
       <c r="M30" s="3" t="n">
-        <v>1159.2</v>
+        <v>152.6</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>23.9</v>
+        <v>123.9</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>487.6</v>
+        <v>95.3</v>
       </c>
       <c r="P30" s="3" t="n">
         <v>2.8</v>
       </c>
       <c r="Q30" s="3" t="n">
-        <v>1185.8</v>
+        <v>35.8</v>
       </c>
       <c r="R30" s="3" t="n">
         <v>120.7</v>
       </c>
       <c r="S30" s="3" t="n">
-        <v>140.9</v>
+        <v>28</v>
       </c>
       <c r="T30" s="3" t="n">
-        <v>396.8</v>
+        <v>22</v>
       </c>
       <c r="U30" s="3" t="n">
-        <v>14.2</v>
+        <v>9.5</v>
       </c>
       <c r="V30" s="3" t="n">
-        <v>126.1</v>
+        <v>22.4</v>
       </c>
       <c r="W30" s="3" t="n">
         <v>21.3</v>
       </c>
       <c r="X30" s="3" t="n">
-        <v>135.8</v>
+        <v>24.6</v>
       </c>
       <c r="Y30" s="3" t="n">
-        <v>90.8</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="Z30" s="3" t="n">
-        <v>2.5</v>
+        <v>25.8</v>
       </c>
       <c r="AA30" s="3" t="inlineStr">
         <is>
@@ -3060,29 +3089,29 @@
       <c r="C31" s="3" t="n">
         <v>211.2</v>
       </c>
-      <c r="D31" s="10" t="n">
-        <v>29</v>
-      </c>
-      <c r="E31" s="10" t="n">
+      <c r="D31" s="3" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="E31" s="3" t="n">
         <v>20.6</v>
       </c>
-      <c r="F31" s="10" t="n">
-        <v>24.8</v>
-      </c>
-      <c r="G31" s="10" t="n">
-        <v>8.4</v>
+      <c r="F31" s="3" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G31" s="3" t="n">
+        <v>28.4</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>96.59999999999999</v>
+        <v>1.3</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>7.1</v>
+        <v>2.1</v>
       </c>
       <c r="J31" s="3" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="K31" s="3" t="n">
-        <v>38.8</v>
+        <v>0.9</v>
+      </c>
+      <c r="K31" s="8" t="n">
+        <v>1117.1</v>
       </c>
       <c r="L31" s="3" t="n">
         <v>21.3</v>
@@ -3090,44 +3119,44 @@
       <c r="M31" s="3" t="n">
         <v>21</v>
       </c>
-      <c r="N31" s="8" t="n">
-        <v>23.9</v>
+      <c r="N31" s="3" t="n">
+        <v>24.8</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>97.5</v>
+        <v>482.6</v>
       </c>
       <c r="P31" s="3" t="n">
         <v>0.6</v>
       </c>
       <c r="Q31" s="3" t="n">
-        <v>27.2</v>
+        <v>97.2</v>
       </c>
       <c r="R31" s="3" t="n">
         <v>24.1</v>
       </c>
-      <c r="S31" s="3" t="n">
+      <c r="S31" s="8" t="n">
+        <v>40.9</v>
+      </c>
+      <c r="T31" s="3" t="n">
+        <v>396.8</v>
+      </c>
+      <c r="U31" s="3" t="n">
+        <v>38.1</v>
+      </c>
+      <c r="V31" s="8" t="n">
+        <v>26.1</v>
+      </c>
+      <c r="W31" s="3" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="X31" s="8" t="n">
         <v>28.2</v>
       </c>
-      <c r="T31" s="3" t="n">
-        <v>79.40000000000001</v>
-      </c>
-      <c r="U31" s="3" t="n">
-        <v>8.9</v>
-      </c>
-      <c r="V31" s="3" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="W31" s="8" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="X31" s="3" t="n">
-        <v>27.2</v>
-      </c>
       <c r="Y31" s="3" t="n">
-        <v>4.2</v>
+        <v>441.7</v>
       </c>
       <c r="Z31" s="3" t="n">
-        <v>5.8</v>
+        <v>5.2</v>
       </c>
       <c r="AA31" s="3" t="inlineStr">
         <is>
@@ -3145,74 +3174,74 @@
       <c r="C32" s="3" t="n">
         <v>384.7</v>
       </c>
-      <c r="D32" s="10" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="E32" s="10" t="n">
+      <c r="D32" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="E32" s="3" t="n">
         <v>19.3</v>
       </c>
-      <c r="F32" s="10" t="n">
-        <v>25.2</v>
-      </c>
-      <c r="G32" s="10" t="n">
-        <v>11.8</v>
+      <c r="F32" s="3" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="G32" s="3" t="n">
+        <v>1.8</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>19.3</v>
+        <v>18</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>11.4</v>
-      </c>
-      <c r="J32" s="8" t="n">
-        <v>14.6</v>
+        <v>0.4</v>
+      </c>
+      <c r="J32" s="3" t="n">
+        <v>4.6</v>
       </c>
       <c r="K32" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="L32" s="8" t="n">
+      <c r="L32" s="3" t="n">
         <v>20.1</v>
       </c>
       <c r="M32" s="3" t="n">
-        <v>20.1</v>
-      </c>
-      <c r="N32" s="8" t="n">
-        <v>24.8</v>
+        <v>26.1</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>2.2</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>100</v>
+        <v>78.5</v>
       </c>
       <c r="P32" s="3" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="Q32" s="3" t="n">
-        <v>31.1</v>
-      </c>
-      <c r="R32" s="8" t="n">
-        <v>24.9</v>
+        <v>34.1</v>
+      </c>
+      <c r="R32" s="3" t="n">
+        <v>43.9</v>
       </c>
       <c r="S32" s="3" t="n">
-        <v>22.5</v>
+        <v>28.2</v>
       </c>
       <c r="T32" s="3" t="n">
-        <v>61</v>
+        <v>9.4</v>
       </c>
       <c r="U32" s="3" t="n">
         <v>17.5</v>
       </c>
       <c r="V32" s="3" t="n">
-        <v>97.40000000000001</v>
+        <v>25.2</v>
       </c>
       <c r="W32" s="3" t="n">
         <v>23.2</v>
       </c>
       <c r="X32" s="3" t="n">
-        <v>27.2</v>
+        <v>92.2</v>
       </c>
       <c r="Y32" s="3" t="n">
         <v>24.9</v>
       </c>
       <c r="Z32" s="3" t="n">
-        <v>5.2</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="AA32" s="3" t="inlineStr">
         <is>
@@ -3228,76 +3257,79 @@
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>213.3</v>
-      </c>
-      <c r="D33" s="10" t="n">
-        <v>29.2</v>
-      </c>
-      <c r="E33" s="10" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="F33" s="10" t="n">
-        <v>24.4</v>
-      </c>
-      <c r="G33" s="10" t="n">
+        <v>242.3</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <v>244.4</v>
+      </c>
+      <c r="G33" s="3" t="n">
         <v>9.6</v>
       </c>
-      <c r="H33" s="8" t="n">
-        <v>18</v>
+      <c r="H33" s="3" t="n">
+        <v>18.8</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>8.300000000000001</v>
+        <v>2.3</v>
       </c>
       <c r="J33" s="3" t="n">
-        <v>51.6</v>
+        <v>1.6</v>
       </c>
       <c r="K33" s="3" t="n">
-        <v>14.8</v>
+        <v>4.9</v>
       </c>
       <c r="L33" s="3" t="n">
         <v>21.5</v>
       </c>
-      <c r="M33" s="8" t="n">
-        <v>21.4</v>
-      </c>
-      <c r="N33" s="8" t="n">
-        <v>23.5</v>
+      <c r="M33" s="3" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>2.2</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>99</v>
+        <v>160</v>
       </c>
       <c r="P33" s="3" t="n">
         <v>0.2</v>
       </c>
       <c r="Q33" s="3" t="n">
-        <v>28.9</v>
-      </c>
-      <c r="R33" s="8" t="n">
-        <v>84.59999999999999</v>
+        <v>2.9</v>
+      </c>
+      <c r="R33" s="3" t="n">
+        <v>4.6</v>
       </c>
       <c r="S33" s="3" t="n">
-        <v>982.1</v>
+        <v>7.5</v>
       </c>
       <c r="T33" s="3" t="n">
-        <v>70.90000000000001</v>
+        <v>61</v>
       </c>
       <c r="U33" s="3" t="n">
-        <v>11.5</v>
+        <v>1.5</v>
       </c>
       <c r="V33" s="3" t="n">
-        <v>25.6</v>
+        <v>2.4</v>
       </c>
       <c r="W33" s="3" t="n">
         <v>23.8</v>
       </c>
-      <c r="X33" s="3" t="n">
-        <v>28.3</v>
+      <c r="X33" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2862 2
+</t>
+        </is>
       </c>
       <c r="Y33" s="3" t="n">
-        <v>74.59999999999999</v>
+        <v>4.6</v>
       </c>
       <c r="Z33" s="3" t="n">
-        <v>9.300000000000001</v>
+        <v>4.5</v>
       </c>
       <c r="AA33" s="3" t="inlineStr">
         <is>
@@ -3315,29 +3347,33 @@
       <c r="C34" s="3" t="n">
         <v>311.6</v>
       </c>
-      <c r="D34" s="10" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="E34" s="10" t="n">
-        <v>21.5</v>
-      </c>
-      <c r="F34" s="10" t="n">
+      <c r="D34" s="3" t="n">
+        <v>29.2</v>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">226
+214
+</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="n">
         <v>26.7</v>
       </c>
-      <c r="G34" s="10" t="n">
+      <c r="G34" s="3" t="n">
         <v>10.5</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>18.8</v>
+        <v>20.2</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>8.300000000000001</v>
+        <v>1</v>
       </c>
       <c r="J34" s="3" t="n">
         <v>3.5</v>
       </c>
       <c r="K34" s="3" t="n">
-        <v>0.2</v>
+        <v>0.8</v>
       </c>
       <c r="L34" s="3" t="n">
         <v>21.8</v>
@@ -3345,44 +3381,44 @@
       <c r="M34" s="3" t="n">
         <v>21.7</v>
       </c>
-      <c r="N34" s="8" t="n">
-        <v>25.4</v>
+      <c r="N34" s="3" t="n">
+        <v>85.90000000000001</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>1199</v>
+        <v>99</v>
       </c>
       <c r="P34" s="3" t="n">
         <v>0.2</v>
       </c>
       <c r="Q34" s="3" t="n">
-        <v>20.5</v>
+        <v>30.5</v>
       </c>
       <c r="R34" s="3" t="n">
         <v>25.8</v>
       </c>
       <c r="S34" s="3" t="n">
-        <v>30.2</v>
+        <v>28.2</v>
       </c>
       <c r="T34" s="3" t="n">
-        <v>69.40000000000001</v>
+        <v>20.9</v>
       </c>
       <c r="U34" s="3" t="n">
         <v>13.3</v>
       </c>
       <c r="V34" s="3" t="n">
-        <v>27.3</v>
-      </c>
-      <c r="W34" s="8" t="n">
-        <v>138248.4</v>
+        <v>25.6</v>
+      </c>
+      <c r="W34" s="3" t="n">
+        <v>23.8</v>
       </c>
       <c r="X34" s="3" t="n">
-        <v>29.7</v>
+        <v>22.8</v>
       </c>
       <c r="Y34" s="3" t="n">
-        <v>262.1</v>
+        <v>4.6</v>
       </c>
       <c r="Z34" s="3" t="n">
-        <v>4.5</v>
+        <v>6.5</v>
       </c>
       <c r="AA34" s="3" t="inlineStr">
         <is>
@@ -3400,29 +3436,29 @@
       <c r="C35" s="3" t="n">
         <v>353.4</v>
       </c>
-      <c r="D35" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="E35" s="10" t="n">
-        <v>20.7</v>
-      </c>
-      <c r="F35" s="10" t="n">
+      <c r="D35" s="3" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>20.8</v>
+      </c>
+      <c r="F35" s="3" t="n">
         <v>25.9</v>
       </c>
-      <c r="G35" s="10" t="n">
+      <c r="G35" s="3" t="n">
         <v>10.3</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>20.2</v>
+        <v>19.7</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>12.4</v>
+        <v>2</v>
       </c>
       <c r="J35" s="3" t="n">
         <v>4</v>
       </c>
       <c r="K35" s="3" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="L35" s="3" t="n">
         <v>21.6</v>
@@ -3431,43 +3467,43 @@
         <v>21.3</v>
       </c>
       <c r="N35" s="3" t="n">
-        <v>25.9</v>
+        <v>85.90000000000001</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>97.8</v>
+        <v>92</v>
       </c>
       <c r="P35" s="3" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="Q35" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="Q35" s="3" t="n">
         <v>31.1</v>
       </c>
       <c r="R35" s="3" t="n">
-        <v>26.9</v>
+        <v>0.2</v>
       </c>
       <c r="S35" s="3" t="n">
-        <v>27.5</v>
+        <v>30.2</v>
       </c>
       <c r="T35" s="3" t="n">
-        <v>61.3</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="U35" s="3" t="n">
-        <v>17.4</v>
+        <v>7.4</v>
       </c>
       <c r="V35" s="3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="W35" s="8" t="n">
-        <v>46.6</v>
+        <v>72.3</v>
+      </c>
+      <c r="W35" s="3" t="n">
+        <v>24.8</v>
       </c>
       <c r="X35" s="3" t="n">
-        <v>28.9</v>
+        <v>8.9</v>
       </c>
       <c r="Y35" s="3" t="n">
-        <v>82</v>
+        <v>4.4</v>
       </c>
       <c r="Z35" s="3" t="n">
-        <v>6.5</v>
+        <v>0.4</v>
       </c>
       <c r="AA35" s="3" t="inlineStr">
         <is>
@@ -3485,44 +3521,44 @@
       <c r="C36" s="3" t="n">
         <v>430.7</v>
       </c>
-      <c r="D36" s="10" t="n">
-        <v>32.1</v>
-      </c>
-      <c r="E36" s="10" t="n">
+      <c r="D36" s="3" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="E36" s="3" t="n">
         <v>20.9</v>
       </c>
-      <c r="F36" s="10" t="n">
+      <c r="F36" s="3" t="n">
         <v>26.5</v>
       </c>
-      <c r="G36" s="10" t="n">
-        <v>11.2</v>
+      <c r="G36" s="3" t="n">
+        <v>1.2</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>19.8</v>
+        <v>12.8</v>
       </c>
       <c r="I36" s="3" t="n">
         <v>2.4</v>
       </c>
       <c r="J36" s="3" t="n">
-        <v>14.4</v>
+        <v>4.4</v>
       </c>
       <c r="K36" s="3" t="n">
         <v>30.6</v>
       </c>
-      <c r="L36" s="8" t="n">
-        <v>41</v>
+      <c r="L36" s="3" t="n">
+        <v>21</v>
       </c>
       <c r="M36" s="3" t="n">
         <v>20.7</v>
       </c>
       <c r="N36" s="3" t="n">
-        <v>25.1</v>
+        <v>4.2</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>972.5</v>
+        <v>97.5</v>
       </c>
       <c r="P36" s="3" t="n">
-        <v>10.6</v>
+        <v>0.6</v>
       </c>
       <c r="Q36" s="3" t="n">
         <v>32.1</v>
@@ -3531,28 +3567,28 @@
         <v>26</v>
       </c>
       <c r="S36" s="3" t="n">
-        <v>29.7</v>
+        <v>7.5</v>
       </c>
       <c r="T36" s="3" t="n">
         <v>62.2</v>
       </c>
-      <c r="U36" s="3" t="n">
-        <v>18</v>
+      <c r="U36" s="8" t="n">
+        <v>82</v>
       </c>
       <c r="V36" s="3" t="n">
-        <v>28.7</v>
-      </c>
-      <c r="W36" s="8" t="n">
+        <v>27.8</v>
+      </c>
+      <c r="W36" s="3" t="n">
         <v>24.6</v>
       </c>
       <c r="X36" s="3" t="n">
         <v>28.3</v>
       </c>
       <c r="Y36" s="3" t="n">
-        <v>79.40000000000001</v>
+        <v>28.3</v>
       </c>
       <c r="Z36" s="3" t="n">
-        <v>8.4</v>
+        <v>0.1</v>
       </c>
       <c r="AA36" s="3" t="inlineStr">
         <is>
@@ -3568,76 +3604,84 @@
         </is>
       </c>
       <c r="C37" s="3" t="n">
-        <v>1693.7</v>
-      </c>
-      <c r="D37" s="10" t="n">
-        <v>155.4</v>
-      </c>
-      <c r="E37" s="10" t="n">
-        <v>102</v>
-      </c>
-      <c r="F37" s="10" t="n">
+        <v>693.7</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F37" s="3" t="n">
         <v>128.7</v>
       </c>
-      <c r="G37" s="10" t="n">
+      <c r="G37" s="3" t="n">
         <v>53.4</v>
       </c>
       <c r="H37" s="3" t="n">
         <v>96.5</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>10.1</v>
+        <v>4</v>
       </c>
       <c r="J37" s="3" t="n">
-        <v>0.4</v>
+        <v>18.1</v>
       </c>
       <c r="K37" s="3" t="n">
         <v>35.6</v>
       </c>
       <c r="L37" s="3" t="n">
-        <v>106</v>
+        <v>16</v>
       </c>
       <c r="M37" s="3" t="n">
-        <v>1015.9</v>
+        <v>15.2</v>
       </c>
       <c r="N37" s="3" t="n">
-        <v>24.2</v>
+        <v>24.1</v>
       </c>
       <c r="O37" s="3" t="n">
-        <v>1192.7</v>
+        <v>42.7</v>
       </c>
       <c r="P37" s="3" t="n">
         <v>1.7</v>
       </c>
       <c r="Q37" s="3" t="n">
-        <v>153.7</v>
+        <v>53.7</v>
       </c>
       <c r="R37" s="3" t="n">
         <v>126.2</v>
       </c>
-      <c r="S37" s="3" t="n">
-        <v>1143.1</v>
+      <c r="S37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">792798
+11811
+</t>
+        </is>
       </c>
       <c r="T37" s="3" t="n">
         <v>324.8</v>
       </c>
       <c r="U37" s="3" t="n">
-        <v>77.7</v>
+        <v>3.7</v>
       </c>
       <c r="V37" s="3" t="n">
-        <v>136.8</v>
+        <v>28.7</v>
       </c>
       <c r="W37" s="3" t="n">
-        <v>121.6</v>
+        <v>46.6</v>
       </c>
       <c r="X37" s="3" t="n">
-        <v>7.2</v>
+        <v>12.4</v>
       </c>
       <c r="Y37" s="3" t="n">
-        <v>72</v>
-      </c>
-      <c r="Z37" s="3" t="n">
-        <v>1.1</v>
+        <v>726</v>
+      </c>
+      <c r="Z37" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">82745857727
+12119
+</t>
+        </is>
       </c>
       <c r="AA37" s="3" t="inlineStr">
         <is>
@@ -3655,74 +3699,74 @@
       <c r="C38" s="3" t="n">
         <v>338.7</v>
       </c>
-      <c r="D38" s="10" t="n">
-        <v>31</v>
-      </c>
-      <c r="E38" s="10" t="n">
-        <v>20.4</v>
-      </c>
-      <c r="F38" s="10" t="n">
-        <v>25.7</v>
-      </c>
-      <c r="G38" s="10" t="n">
+      <c r="D38" s="3" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="G38" s="3" t="n">
         <v>10.6</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>19.3</v>
+        <v>2.3</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J38" s="3" t="n">
-        <v>18.1</v>
+        <v>3.6</v>
       </c>
       <c r="K38" s="3" t="n">
         <v>35.6</v>
       </c>
       <c r="L38" s="3" t="n">
-        <v>21.2</v>
-      </c>
-      <c r="M38" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="N38" s="8" t="n">
-        <v>28.1</v>
+        <v>41.2</v>
+      </c>
+      <c r="M38" s="8" t="n">
+        <v>41</v>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>4.8</v>
       </c>
       <c r="O38" s="3" t="n">
         <v>98.5</v>
       </c>
       <c r="P38" s="3" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Q38" s="3" t="n">
-        <v>20.7</v>
+        <v>9.300000000000001</v>
+      </c>
+      <c r="Q38" s="8" t="n">
+        <v>60.7</v>
       </c>
       <c r="R38" s="3" t="n">
         <v>25.2</v>
       </c>
-      <c r="S38" s="3" t="n">
-        <v>28.6</v>
+      <c r="S38" s="8" t="n">
+        <v>43.1</v>
       </c>
       <c r="T38" s="3" t="n">
-        <v>65</v>
+        <v>6</v>
       </c>
       <c r="U38" s="3" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="V38" s="3" t="n">
-        <v>87.40000000000001</v>
-      </c>
-      <c r="W38" s="3" t="n">
-        <v>24.3</v>
-      </c>
-      <c r="X38" s="3" t="n">
-        <v>28.5</v>
+        <v>2.5</v>
+      </c>
+      <c r="V38" s="8" t="n">
+        <v>36.8</v>
+      </c>
+      <c r="W38" s="8" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="X38" s="8" t="n">
+        <v>92.2</v>
       </c>
       <c r="Y38" s="3" t="n">
-        <v>98.2</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="Z38" s="3" t="n">
-        <v>1.9</v>
+        <v>39.7</v>
       </c>
       <c r="AA38" s="3" t="inlineStr">
         <is>
@@ -3738,76 +3782,80 @@
         </is>
       </c>
       <c r="C39" s="3" t="n">
-        <v>332.5</v>
-      </c>
-      <c r="D39" s="10" t="n">
-        <v>31.9</v>
-      </c>
-      <c r="E39" s="10" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="F39" s="10" t="n">
+        <v>32.5</v>
+      </c>
+      <c r="D39" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="E39" s="3" t="n">
+        <v>90.09999999999999</v>
+      </c>
+      <c r="F39" s="3" t="n">
         <v>26.1</v>
       </c>
-      <c r="G39" s="10" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="H39" s="8" t="n">
+      <c r="G39" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="H39" s="3" t="n">
         <v>19.3</v>
       </c>
       <c r="I39" s="3" t="n">
         <v>1.7</v>
       </c>
       <c r="J39" s="3" t="n">
-        <v>3.6</v>
+        <v>3</v>
       </c>
       <c r="K39" s="3" t="n">
-        <v>0.6</v>
+        <v>8.9</v>
       </c>
       <c r="L39" s="3" t="n">
-        <v>28</v>
-      </c>
-      <c r="M39" s="8" t="n">
-        <v>20.9</v>
-      </c>
-      <c r="N39" s="8" t="n">
-        <v>14.8</v>
+        <v>84</v>
+      </c>
+      <c r="M39" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">269
+111
+</t>
+        </is>
+      </c>
+      <c r="N39" s="3" t="n">
+        <v>20.6</v>
       </c>
       <c r="O39" s="3" t="n">
         <v>99</v>
       </c>
       <c r="P39" s="3" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="Q39" s="3" t="n">
-        <v>71.90000000000001</v>
+        <v>31.9</v>
       </c>
       <c r="R39" s="3" t="n">
-        <v>86</v>
+        <v>26</v>
       </c>
       <c r="S39" s="3" t="n">
-        <v>89.8</v>
+        <v>28.6</v>
       </c>
       <c r="T39" s="3" t="n">
         <v>63.2</v>
       </c>
       <c r="U39" s="3" t="n">
-        <v>17.3</v>
+        <v>12.3</v>
       </c>
       <c r="V39" s="3" t="n">
-        <v>24.7</v>
+        <v>28.4</v>
       </c>
       <c r="W39" s="3" t="n">
-        <v>23.2</v>
+        <v>24.3</v>
       </c>
       <c r="X39" s="3" t="n">
-        <v>27.6</v>
+        <v>28.5</v>
       </c>
       <c r="Y39" s="3" t="n">
-        <v>78.40000000000001</v>
+        <v>88.2</v>
       </c>
       <c r="Z39" s="3" t="n">
-        <v>38.6</v>
+        <v>2.9</v>
       </c>
       <c r="AA39" s="3" t="inlineStr">
         <is>
@@ -3822,29 +3870,33 @@
           <t>27</t>
         </is>
       </c>
-      <c r="C40" s="3" t="n">
-        <v>453.7</v>
-      </c>
-      <c r="D40" s="10" t="n">
-        <v>32.9</v>
-      </c>
-      <c r="E40" s="10" t="n">
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7924
+265
+</t>
+        </is>
+      </c>
+      <c r="D40" s="8" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="E40" s="3" t="n">
         <v>18.8</v>
       </c>
-      <c r="F40" s="10" t="n">
+      <c r="F40" s="3" t="n">
         <v>25.9</v>
       </c>
-      <c r="G40" s="10" t="n">
-        <v>14.1</v>
-      </c>
-      <c r="H40" s="8" t="n">
+      <c r="G40" s="3" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="H40" s="3" t="n">
         <v>18.2</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>12.7</v>
+        <v>2.7</v>
       </c>
       <c r="J40" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K40" s="3" t="n">
         <v>0</v>
@@ -3852,17 +3904,21 @@
       <c r="L40" s="3" t="n">
         <v>19.8</v>
       </c>
-      <c r="M40" s="3" t="n">
-        <v>19.6</v>
-      </c>
-      <c r="N40" s="8" t="n">
-        <v>46.8</v>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">269
+111
+</t>
+        </is>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>2.6</v>
       </c>
       <c r="O40" s="3" t="n">
         <v>97.8</v>
       </c>
       <c r="P40" s="3" t="n">
-        <v>0.5</v>
+        <v>6.5</v>
       </c>
       <c r="Q40" s="3" t="n">
         <v>32.8</v>
@@ -3870,29 +3926,29 @@
       <c r="R40" s="3" t="n">
         <v>26</v>
       </c>
-      <c r="S40" s="8" t="n">
-        <v>29.3</v>
+      <c r="S40" s="3" t="n">
+        <v>22.8</v>
       </c>
       <c r="T40" s="3" t="n">
-        <v>59.2</v>
+        <v>2.6</v>
       </c>
       <c r="U40" s="3" t="n">
-        <v>20.2</v>
+        <v>2.6</v>
       </c>
       <c r="V40" s="3" t="n">
-        <v>27.8</v>
+        <v>24.2</v>
       </c>
       <c r="W40" s="3" t="n">
-        <v>23.8</v>
+        <v>2.2</v>
       </c>
       <c r="X40" s="3" t="n">
-        <v>26.9</v>
+        <v>2.5</v>
       </c>
       <c r="Y40" s="3" t="n">
-        <v>98.2</v>
+        <v>7.1</v>
       </c>
       <c r="Z40" s="3" t="n">
-        <v>10.4</v>
+        <v>3.6</v>
       </c>
       <c r="AA40" s="3" t="inlineStr">
         <is>
@@ -3907,41 +3963,45 @@
           <t>28</t>
         </is>
       </c>
-      <c r="C41" s="3" t="n">
-        <v>265.6</v>
-      </c>
-      <c r="D41" s="10" t="n">
-        <v>31.6</v>
-      </c>
-      <c r="E41" s="10" t="n">
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">7924
+265
+</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="n">
+        <v>32.9</v>
+      </c>
+      <c r="E41" s="3" t="n">
         <v>19.6</v>
       </c>
-      <c r="F41" s="10" t="n">
+      <c r="F41" s="3" t="n">
         <v>25.6</v>
       </c>
-      <c r="G41" s="10" t="n">
+      <c r="G41" s="3" t="n">
         <v>12</v>
       </c>
-      <c r="H41" s="8" t="n">
-        <v>18</v>
+      <c r="H41" s="3" t="n">
+        <v>18.1</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>11.2</v>
+        <v>1.2</v>
       </c>
       <c r="J41" s="3" t="n">
-        <v>5</v>
+        <v>1.6</v>
       </c>
       <c r="K41" s="3" t="n">
-        <v>43.4</v>
+        <v>0</v>
       </c>
       <c r="L41" s="3" t="n">
-        <v>19.9</v>
+        <v>9.9</v>
       </c>
       <c r="M41" s="3" t="n">
         <v>19.8</v>
       </c>
-      <c r="N41" s="8" t="n">
-        <v>28.6</v>
+      <c r="N41" s="3" t="n">
+        <v>23</v>
       </c>
       <c r="O41" s="3" t="n">
         <v>99</v>
@@ -3956,28 +4016,28 @@
         <v>21.4</v>
       </c>
       <c r="S41" s="3" t="n">
-        <v>24.9</v>
+        <v>29.3</v>
       </c>
       <c r="T41" s="3" t="n">
-        <v>92.3</v>
+        <v>22.3</v>
       </c>
       <c r="U41" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="V41" s="8" t="n">
-        <v>28.1</v>
+      <c r="V41" s="3" t="n">
+        <v>2.8</v>
       </c>
       <c r="W41" s="3" t="n">
-        <v>23.4</v>
+        <v>23.8</v>
       </c>
       <c r="X41" s="3" t="n">
-        <v>28</v>
+        <v>2.5</v>
       </c>
       <c r="Y41" s="3" t="n">
-        <v>22</v>
+        <v>29.6</v>
       </c>
       <c r="Z41" s="3" t="n">
-        <v>8.9</v>
+        <v>1.4</v>
       </c>
       <c r="AA41" s="3" t="inlineStr">
         <is>
@@ -3995,44 +4055,44 @@
       <c r="C42" s="3" t="n">
         <v>236.3</v>
       </c>
-      <c r="D42" s="10" t="n">
+      <c r="D42" s="3" t="n">
         <v>31.6</v>
       </c>
-      <c r="E42" s="10" t="n">
+      <c r="E42" s="3" t="n">
         <v>20.3</v>
       </c>
-      <c r="F42" s="10" t="n">
+      <c r="F42" s="3" t="n">
         <v>25.9</v>
       </c>
-      <c r="G42" s="10" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="H42" s="8" t="n">
-        <v>20</v>
+      <c r="G42" s="3" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>26</v>
       </c>
       <c r="I42" s="3" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="J42" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="K42" s="3" t="n">
         <v>0.7</v>
       </c>
-      <c r="J42" s="3" t="n">
-        <v>1.6</v>
-      </c>
-      <c r="K42" s="3" t="n">
-        <v>28.7</v>
-      </c>
       <c r="L42" s="3" t="n">
-        <v>21.9</v>
-      </c>
-      <c r="M42" s="8" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="M42" s="3" t="n">
         <v>21.8</v>
       </c>
       <c r="N42" s="3" t="n">
-        <v>83</v>
+        <v>26</v>
       </c>
       <c r="O42" s="3" t="n">
-        <v>199</v>
+        <v>99</v>
       </c>
       <c r="P42" s="3" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="Q42" s="3" t="n">
         <v>24.1</v>
@@ -4041,28 +4101,28 @@
         <v>23.8</v>
       </c>
       <c r="S42" s="3" t="n">
-        <v>89.3</v>
+        <v>24.9</v>
       </c>
       <c r="T42" s="3" t="n">
-        <v>97.7</v>
+        <v>92.2</v>
       </c>
       <c r="U42" s="3" t="n">
-        <v>0.7</v>
+        <v>2.7</v>
       </c>
       <c r="V42" s="3" t="n">
-        <v>85.90000000000001</v>
+        <v>24.6</v>
       </c>
       <c r="W42" s="3" t="n">
-        <v>23.5</v>
+        <v>23.4</v>
       </c>
       <c r="X42" s="3" t="n">
-        <v>28.2</v>
+        <v>2.7</v>
       </c>
       <c r="Y42" s="3" t="n">
-        <v>90.59999999999999</v>
+        <v>29.6</v>
       </c>
       <c r="Z42" s="3" t="n">
-        <v>8.9</v>
+        <v>2.9</v>
       </c>
       <c r="AA42" s="3" t="inlineStr">
         <is>
@@ -4078,40 +4138,40 @@
         </is>
       </c>
       <c r="C43" s="3" t="n">
-        <v>372.2</v>
-      </c>
-      <c r="D43" s="10" t="n">
-        <v>30</v>
-      </c>
-      <c r="E43" s="10" t="n">
+        <v>72.2</v>
+      </c>
+      <c r="D43" s="3" t="n">
+        <v>31.6</v>
+      </c>
+      <c r="E43" s="3" t="n">
         <v>21.3</v>
       </c>
-      <c r="F43" s="10" t="n">
-        <v>25.6</v>
-      </c>
-      <c r="G43" s="10" t="n">
+      <c r="F43" s="3" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="G43" s="3" t="n">
         <v>8.699999999999999</v>
       </c>
-      <c r="H43" s="8" t="n">
+      <c r="H43" s="3" t="n">
         <v>19.8</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="J43" s="3" t="n">
         <v>1.5</v>
       </c>
       <c r="K43" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="L43" s="3" t="n">
         <v>21.6</v>
       </c>
       <c r="M43" s="3" t="n">
-        <v>21.5</v>
+        <v>24.5</v>
       </c>
       <c r="N43" s="3" t="n">
-        <v>95.59999999999999</v>
+        <v>354.6</v>
       </c>
       <c r="O43" s="3" t="n">
         <v>99</v>
@@ -4123,31 +4183,31 @@
         <v>29.1</v>
       </c>
       <c r="R43" s="3" t="n">
-        <v>25.5</v>
+        <v>23.8</v>
       </c>
       <c r="S43" s="3" t="n">
-        <v>30.4</v>
+        <v>29.3</v>
       </c>
       <c r="T43" s="3" t="n">
         <v>75.59999999999999</v>
       </c>
       <c r="U43" s="3" t="n">
-        <v>9.800000000000001</v>
+        <v>2.8</v>
       </c>
       <c r="V43" s="3" t="n">
-        <v>27.8</v>
-      </c>
-      <c r="W43" s="3" t="n">
-        <v>84.7</v>
+        <v>2.7</v>
+      </c>
+      <c r="W43" s="8" t="n">
+        <v>23.5</v>
       </c>
       <c r="X43" s="3" t="n">
-        <v>9.1</v>
+        <v>2.1</v>
       </c>
       <c r="Y43" s="3" t="n">
-        <v>78</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="Z43" s="3" t="n">
-        <v>9.199999999999999</v>
+        <v>0.5</v>
       </c>
       <c r="AA43" s="3" t="inlineStr">
         <is>
@@ -4165,17 +4225,17 @@
       <c r="C44" s="3" t="n">
         <v>365.9</v>
       </c>
-      <c r="D44" s="10" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="E44" s="10" t="n">
+      <c r="D44" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="E44" s="3" t="n">
         <v>21.3</v>
       </c>
-      <c r="F44" s="10" t="n">
+      <c r="F44" s="3" t="n">
         <v>26.9</v>
       </c>
-      <c r="G44" s="10" t="n">
-        <v>11.3</v>
+      <c r="G44" s="3" t="n">
+        <v>1.3</v>
       </c>
       <c r="H44" s="3" t="n">
         <v>19.4</v>
@@ -4190,49 +4250,49 @@
         <v>0</v>
       </c>
       <c r="L44" s="3" t="n">
-        <v>22.3</v>
+        <v>28.3</v>
       </c>
       <c r="M44" s="3" t="n">
-        <v>82.3</v>
+        <v>2.3</v>
       </c>
       <c r="N44" s="3" t="n">
         <v>26.9</v>
       </c>
       <c r="O44" s="3" t="n">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="P44" s="3" t="n">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="Q44" s="3" t="n">
-        <v>22.6</v>
+        <v>32.6</v>
       </c>
       <c r="R44" s="3" t="n">
-        <v>26.4</v>
+        <v>66.8</v>
       </c>
       <c r="S44" s="3" t="n">
-        <v>30.4</v>
+        <v>24.8</v>
       </c>
       <c r="T44" s="3" t="n">
-        <v>62</v>
+        <v>62.1</v>
       </c>
       <c r="U44" s="3" t="n">
         <v>18.6</v>
       </c>
       <c r="V44" s="3" t="n">
-        <v>88.5</v>
+        <v>46.2</v>
       </c>
       <c r="W44" s="3" t="n">
-        <v>26.3</v>
+        <v>24.7</v>
       </c>
       <c r="X44" s="3" t="n">
-        <v>22.8</v>
+        <v>32.8</v>
       </c>
       <c r="Y44" s="3" t="n">
-        <v>84.40000000000001</v>
+        <v>84.09999999999999</v>
       </c>
       <c r="Z44" s="3" t="n">
-        <v>6</v>
+        <v>2.2</v>
       </c>
       <c r="AA44" s="3" t="inlineStr">
         <is>
@@ -4248,77 +4308,71 @@
         </is>
       </c>
       <c r="C45" s="3" t="n">
-        <v>20.8</v>
-      </c>
-      <c r="D45" s="10" t="n">
-        <v>190.6</v>
-      </c>
-      <c r="E45" s="10" t="n">
-        <v>121.6</v>
-      </c>
-      <c r="F45" s="10" t="n">
-        <v>156.1</v>
-      </c>
-      <c r="G45" s="10" t="n">
-        <v>69.09999999999999</v>
+        <v>2.2</v>
+      </c>
+      <c r="D45" s="3" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="E45" s="3" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F45" s="3" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="G45" s="3" t="n">
+        <v>3.7</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>427.4</v>
+        <v>14.7</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>1.9</v>
+        <v>1.2</v>
       </c>
       <c r="J45" s="3" t="n">
-        <v>18.8</v>
+        <v>28.9</v>
       </c>
       <c r="K45" s="3" t="n">
-        <v>0</v>
+        <v>728.3</v>
       </c>
       <c r="L45" s="3" t="n">
-        <v>22.3</v>
+        <v>726.3</v>
       </c>
       <c r="M45" s="3" t="n">
-        <v>1825.9</v>
+        <v>3.9</v>
       </c>
       <c r="N45" s="3" t="n">
-        <v>26.9</v>
+        <v>98.7</v>
       </c>
       <c r="O45" s="3" t="n">
-        <v>5983.8</v>
+        <v>93.8</v>
       </c>
       <c r="P45" s="3" t="n">
-        <v>1.3</v>
+        <v>2.3</v>
       </c>
       <c r="Q45" s="3" t="n">
-        <v>172.8</v>
-      </c>
-      <c r="R45" s="3" t="n">
-        <v>29.7</v>
-      </c>
-      <c r="S45" s="3" t="n">
-        <v>0.7</v>
-      </c>
+        <v>22.8</v>
+      </c>
+      <c r="R45" s="3" t="n"/>
+      <c r="S45" s="3" t="n"/>
       <c r="T45" s="3" t="n">
-        <v>5</v>
+        <v>450</v>
       </c>
       <c r="U45" s="3" t="n">
-        <v>25.8</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="V45" s="3" t="n">
-        <v>5.8</v>
+        <v>358.1</v>
       </c>
       <c r="W45" s="3" t="n">
-        <v>144.9</v>
+        <v>26.3</v>
       </c>
       <c r="X45" s="3" t="n">
-        <v>77.5</v>
+        <v>172.5</v>
       </c>
       <c r="Y45" s="3" t="n">
-        <v>503.7</v>
-      </c>
-      <c r="Z45" s="3" t="n">
-        <v>8</v>
-      </c>
+        <v>6.2</v>
+      </c>
+      <c r="Z45" s="3" t="n"/>
       <c r="AA45" s="3" t="inlineStr">
         <is>
           <t>Tot.</t>
@@ -4333,19 +4387,19 @@
         </is>
       </c>
       <c r="C46" s="3" t="n">
-        <v>237.6</v>
-      </c>
-      <c r="D46" s="10" t="n">
-        <v>31.7</v>
-      </c>
-      <c r="E46" s="10" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="F46" s="10" t="n">
-        <v>25.9</v>
-      </c>
-      <c r="G46" s="10" t="n">
-        <v>11.5</v>
+        <v>37.6</v>
+      </c>
+      <c r="D46" s="3" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="E46" s="3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="G46" s="3" t="n">
+        <v>1.5</v>
       </c>
       <c r="H46" s="3" t="n">
         <v>19.1</v>
@@ -4356,52 +4410,52 @@
       <c r="J46" s="3" t="n">
         <v>3.1</v>
       </c>
-      <c r="K46" s="3" t="n"/>
+      <c r="K46" s="8" t="n">
+        <v>28.3</v>
+      </c>
       <c r="L46" s="3" t="n">
-        <v>21.1</v>
+        <v>41.1</v>
       </c>
       <c r="M46" s="3" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="N46" s="3" t="n">
-        <v>84.8</v>
+        <v>24.8</v>
       </c>
       <c r="O46" s="3" t="n">
         <v>99</v>
       </c>
       <c r="P46" s="3" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
       <c r="Q46" s="3" t="n">
         <v>28.8</v>
       </c>
       <c r="R46" s="3" t="n">
-        <v>21.8</v>
+        <v>4.8</v>
       </c>
       <c r="S46" s="3" t="n">
         <v>29</v>
       </c>
       <c r="T46" s="3" t="n">
-        <v>75</v>
+        <v>28</v>
       </c>
       <c r="U46" s="3" t="n">
-        <v>11.4</v>
+        <v>1.4</v>
       </c>
       <c r="V46" s="3" t="n">
-        <v>26.3</v>
+        <v>6.3</v>
       </c>
       <c r="W46" s="8" t="n">
-        <v>14.1</v>
+        <v>44.2</v>
       </c>
       <c r="X46" s="3" t="n">
         <v>28.7</v>
       </c>
       <c r="Y46" s="3" t="n">
-        <v>23.9</v>
-      </c>
-      <c r="Z46" s="3" t="n">
-        <v>5.7</v>
-      </c>
+        <v>23.7</v>
+      </c>
+      <c r="Z46" s="3" t="n"/>
       <c r="AA46" s="3" t="inlineStr">
         <is>
           <t>Moy.</t>

</xml_diff>

<commit_message>
results from updated QA/QC for dry and wet bulb temperatures and humidity
</commit_message>
<xml_diff>
--- a/results/02_post_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_post_QA_QC.xlsx
+++ b/results/02_post_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_post_QA_QC.xlsx
@@ -140,7 +140,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -799,7 +799,7 @@
         <v>28.7</v>
       </c>
       <c r="R4" s="8" t="n">
-        <v>22.4</v>
+        <v>24.1</v>
       </c>
       <c r="S4" s="8" t="n">
         <v>27.1</v>
@@ -814,7 +814,7 @@
         <v>25.2</v>
       </c>
       <c r="W4" s="8" t="n">
-        <v>21.9</v>
+        <v>22.8</v>
       </c>
       <c r="X4" s="8" t="n">
         <v>26.2</v>
@@ -884,7 +884,7 @@
         <v>32.6</v>
       </c>
       <c r="R5" s="8" t="n">
-        <v>22.8</v>
+        <v>25.4</v>
       </c>
       <c r="S5" s="8" t="n">
         <v>27.8</v>
@@ -902,13 +902,13 @@
         <v>24</v>
       </c>
       <c r="X5" s="8" t="n">
-        <v>29.8</v>
+        <v>27.6</v>
       </c>
       <c r="Y5" s="8" t="n">
-        <v>82.7</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="Z5" s="8" t="n">
-        <v>6.2</v>
+        <v>8.4</v>
       </c>
       <c r="AA5" s="3" t="inlineStr">
         <is>
@@ -972,19 +972,19 @@
         <v>25.7</v>
       </c>
       <c r="S6" s="8" t="n">
-        <v>33</v>
+        <v>28.2</v>
       </c>
       <c r="T6" s="8" t="n">
-        <v>66.7</v>
+        <v>57</v>
       </c>
       <c r="U6" s="8" t="n">
-        <v>16.5</v>
+        <v>21.3</v>
       </c>
       <c r="V6" s="8" t="n">
         <v>28.7</v>
       </c>
       <c r="W6" s="8" t="n">
-        <v>21.8</v>
+        <v>23.7</v>
       </c>
       <c r="X6" s="8" t="n">
         <v>26.1</v>
@@ -1054,7 +1054,7 @@
         <v>34.2</v>
       </c>
       <c r="R7" s="8" t="n">
-        <v>22.4</v>
+        <v>25.5</v>
       </c>
       <c r="S7" s="8" t="n">
         <v>27.1</v>
@@ -1072,13 +1072,13 @@
         <v>24.4</v>
       </c>
       <c r="X7" s="8" t="n">
-        <v>30.6</v>
+        <v>27.1</v>
       </c>
       <c r="Y7" s="8" t="n">
-        <v>74.09999999999999</v>
+        <v>65.59999999999999</v>
       </c>
       <c r="Z7" s="8" t="n">
-        <v>10.7</v>
+        <v>14.2</v>
       </c>
       <c r="AA7" s="3" t="inlineStr">
         <is>
@@ -1127,13 +1127,13 @@
         <v>20.6</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>24.3</v>
+        <v>24</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>97.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="Q8" s="8" t="n">
         <v>21.4</v>
@@ -1142,13 +1142,13 @@
         <v>21.2</v>
       </c>
       <c r="S8" s="8" t="n">
-        <v>25.2</v>
+        <v>25</v>
       </c>
       <c r="T8" s="8" t="n">
-        <v>98.8</v>
+        <v>98.2</v>
       </c>
       <c r="U8" s="8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="V8" s="8" t="n">
         <v>22.2</v>
@@ -1157,13 +1157,13 @@
         <v>21.9</v>
       </c>
       <c r="X8" s="8" t="n">
-        <v>26.3</v>
+        <v>26.1</v>
       </c>
       <c r="Y8" s="8" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="Z8" s="8" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="AA8" s="3" t="inlineStr">
         <is>
@@ -1223,7 +1223,7 @@
       <c r="Q9" s="8" t="n">
         <v>149.6</v>
       </c>
-      <c r="R9" s="9" t="n">
+      <c r="R9" s="8" t="n">
         <v>121.9</v>
       </c>
       <c r="S9" s="3" t="n">
@@ -1238,7 +1238,7 @@
       <c r="V9" s="8" t="n">
         <v>132.8</v>
       </c>
-      <c r="W9" s="9" t="n">
+      <c r="W9" s="8" t="n">
         <v>116.8</v>
       </c>
       <c r="X9" s="3" t="n">
@@ -1298,40 +1298,40 @@
         <v>23.2</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>99.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="Q10" s="8" t="n">
         <v>29.9</v>
       </c>
-      <c r="R10" s="9" t="n">
+      <c r="R10" s="8" t="n">
         <v>24.4</v>
       </c>
       <c r="S10" s="8" t="n">
-        <v>30.6</v>
+        <v>26.8</v>
       </c>
       <c r="T10" s="8" t="n">
-        <v>72.40000000000001</v>
+        <v>63.4</v>
       </c>
       <c r="U10" s="8" t="n">
-        <v>11.7</v>
+        <v>15.4</v>
       </c>
       <c r="V10" s="8" t="n">
         <v>26.6</v>
       </c>
-      <c r="W10" s="9" t="n">
+      <c r="W10" s="8" t="n">
         <v>23.4</v>
       </c>
       <c r="X10" s="8" t="n">
-        <v>28.8</v>
+        <v>26.6</v>
       </c>
       <c r="Y10" s="8" t="n">
-        <v>82.59999999999999</v>
+        <v>76.3</v>
       </c>
       <c r="Z10" s="8" t="n">
-        <v>6.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="AA10" s="3" t="inlineStr">
         <is>
@@ -1380,19 +1380,19 @@
         <v>20.9</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>24.7</v>
+        <v>24.5</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>98.2</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="Q11" s="8" t="n">
         <v>29.9</v>
       </c>
       <c r="R11" s="8" t="n">
-        <v>24</v>
+        <v>25.5</v>
       </c>
       <c r="S11" s="8" t="n">
         <v>29.8</v>
@@ -1407,7 +1407,7 @@
         <v>27.1</v>
       </c>
       <c r="W11" s="8" t="n">
-        <v>24.1</v>
+        <v>24.9</v>
       </c>
       <c r="X11" s="8" t="n">
         <v>30.1</v>
@@ -1465,19 +1465,19 @@
         <v>23</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>28.1</v>
+        <v>27.9</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>98.2</v>
+        <v>97.5</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="Q12" s="8" t="n">
         <v>31.8</v>
       </c>
       <c r="R12" s="8" t="n">
-        <v>22.4</v>
+        <v>24.9</v>
       </c>
       <c r="S12" s="8" t="n">
         <v>27.1</v>
@@ -1492,7 +1492,7 @@
         <v>27.9</v>
       </c>
       <c r="W12" s="8" t="n">
-        <v>23.4</v>
+        <v>24.6</v>
       </c>
       <c r="X12" s="8" t="n">
         <v>28.8</v>
@@ -1550,19 +1550,19 @@
         <v>21.9</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>26.3</v>
+        <v>26.1</v>
       </c>
       <c r="O13" s="8" t="n">
-        <v>98.8</v>
+        <v>98.3</v>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="Q13" s="8" t="n">
         <v>32.6</v>
       </c>
       <c r="R13" s="8" t="n">
-        <v>21.6</v>
+        <v>24.6</v>
       </c>
       <c r="S13" s="8" t="n">
         <v>25.8</v>
@@ -1577,7 +1577,7 @@
         <v>28</v>
       </c>
       <c r="W13" s="8" t="n">
-        <v>23.7</v>
+        <v>24.8</v>
       </c>
       <c r="X13" s="8" t="n">
         <v>29.3</v>
@@ -1650,13 +1650,13 @@
         <v>21.1</v>
       </c>
       <c r="S14" s="8" t="n">
-        <v>25</v>
+        <v>24.1</v>
       </c>
       <c r="T14" s="8" t="n">
-        <v>92.40000000000001</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="U14" s="8" t="n">
-        <v>2.1</v>
+        <v>3</v>
       </c>
       <c r="V14" s="8" t="n">
         <v>22</v>
@@ -1665,13 +1665,13 @@
         <v>21.6</v>
       </c>
       <c r="X14" s="8" t="n">
-        <v>25.8</v>
+        <v>25.5</v>
       </c>
       <c r="Y14" s="8" t="n">
-        <v>97.59999999999999</v>
+        <v>96.5</v>
       </c>
       <c r="Z14" s="8" t="n">
-        <v>0.6</v>
+        <v>0.9</v>
       </c>
       <c r="AA14" s="3" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         <v>32</v>
       </c>
       <c r="R15" s="8" t="n">
-        <v>23.6</v>
+        <v>25.8</v>
       </c>
       <c r="S15" s="8" t="n">
         <v>29.2</v>
@@ -1747,7 +1747,7 @@
         <v>28.7</v>
       </c>
       <c r="W15" s="8" t="n">
-        <v>23.4</v>
+        <v>24.8</v>
       </c>
       <c r="X15" s="8" t="n">
         <v>28.8</v>
@@ -1816,7 +1816,7 @@
       <c r="Q16" s="8" t="n">
         <v>148.7</v>
       </c>
-      <c r="R16" s="9" t="n">
+      <c r="R16" s="8" t="n">
         <v>121.9</v>
       </c>
       <c r="S16" s="3" t="n">
@@ -1831,7 +1831,7 @@
       <c r="V16" s="8" t="n">
         <v>133.7</v>
       </c>
-      <c r="W16" s="9" t="n">
+      <c r="W16" s="8" t="n">
         <v>120.7</v>
       </c>
       <c r="X16" s="3" t="n">
@@ -1890,43 +1890,43 @@
         <v>21.9</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>26.3</v>
+        <v>26.1</v>
       </c>
       <c r="O17" s="8" t="n">
-        <v>98.8</v>
+        <v>98.3</v>
       </c>
       <c r="P17" s="8" t="n">
-        <v>0.3</v>
+        <v>0.5</v>
       </c>
       <c r="Q17" s="8" t="n">
         <v>29.7</v>
       </c>
-      <c r="R17" s="9" t="n">
+      <c r="R17" s="8" t="n">
         <v>24.4</v>
       </c>
       <c r="S17" s="8" t="n">
-        <v>30.6</v>
+        <v>26.9</v>
       </c>
       <c r="T17" s="8" t="n">
-        <v>73.2</v>
+        <v>64.5</v>
       </c>
       <c r="U17" s="8" t="n">
-        <v>11.2</v>
+        <v>14.8</v>
       </c>
       <c r="V17" s="8" t="n">
         <v>26.7</v>
       </c>
-      <c r="W17" s="9" t="n">
+      <c r="W17" s="8" t="n">
         <v>24.1</v>
       </c>
       <c r="X17" s="8" t="n">
-        <v>30</v>
+        <v>28.2</v>
       </c>
       <c r="Y17" s="8" t="n">
-        <v>85.7</v>
+        <v>80.59999999999999</v>
       </c>
       <c r="Z17" s="8" t="n">
-        <v>5</v>
+        <v>6.8</v>
       </c>
       <c r="AA17" s="3" t="inlineStr">
         <is>
@@ -1987,7 +1987,7 @@
         <v>32.1</v>
       </c>
       <c r="R18" s="8" t="n">
-        <v>22.8</v>
+        <v>25.2</v>
       </c>
       <c r="S18" s="8" t="n">
         <v>27.7</v>
@@ -2002,7 +2002,7 @@
         <v>28.5</v>
       </c>
       <c r="W18" s="8" t="n">
-        <v>22.9</v>
+        <v>24.4</v>
       </c>
       <c r="X18" s="8" t="n">
         <v>27.9</v>
@@ -2072,7 +2072,7 @@
         <v>29.9</v>
       </c>
       <c r="R19" s="8" t="n">
-        <v>24.7</v>
+        <v>26</v>
       </c>
       <c r="S19" s="8" t="n">
         <v>31.1</v>
@@ -2087,7 +2087,7 @@
         <v>24.3</v>
       </c>
       <c r="W19" s="8" t="n">
-        <v>22.4</v>
+        <v>22.9</v>
       </c>
       <c r="X19" s="8" t="n">
         <v>27.1</v>
@@ -2157,7 +2157,7 @@
         <v>30.7</v>
       </c>
       <c r="R20" s="8" t="n">
-        <v>22.7</v>
+        <v>24.8</v>
       </c>
       <c r="S20" s="8" t="n">
         <v>27.5</v>
@@ -2172,7 +2172,7 @@
         <v>27.3</v>
       </c>
       <c r="W20" s="8" t="n">
-        <v>22.5</v>
+        <v>23.8</v>
       </c>
       <c r="X20" s="8" t="n">
         <v>27.2</v>
@@ -2242,7 +2242,7 @@
         <v>30.6</v>
       </c>
       <c r="R21" s="8" t="n">
-        <v>24.7</v>
+        <v>26.2</v>
       </c>
       <c r="S21" s="8" t="n">
         <v>31.2</v>
@@ -2257,7 +2257,7 @@
         <v>27.8</v>
       </c>
       <c r="W21" s="8" t="n">
-        <v>23.5</v>
+        <v>24.6</v>
       </c>
       <c r="X21" s="8" t="n">
         <v>28.9</v>
@@ -2327,7 +2327,7 @@
         <v>32.4</v>
       </c>
       <c r="R22" s="8" t="n">
-        <v>23.7</v>
+        <v>25.9</v>
       </c>
       <c r="S22" s="8" t="n">
         <v>29.3</v>
@@ -2342,7 +2342,7 @@
         <v>26.5</v>
       </c>
       <c r="W22" s="8" t="n">
-        <v>23.9</v>
+        <v>24.6</v>
       </c>
       <c r="X22" s="8" t="n">
         <v>29.7</v>
@@ -2411,7 +2411,7 @@
       <c r="Q23" s="8" t="n">
         <v>155.7</v>
       </c>
-      <c r="R23" s="9" t="n">
+      <c r="R23" s="8" t="n">
         <v>128.1</v>
       </c>
       <c r="S23" s="3" t="n">
@@ -2426,7 +2426,7 @@
       <c r="V23" s="8" t="n">
         <v>134.4</v>
       </c>
-      <c r="W23" s="9" t="n">
+      <c r="W23" s="8" t="n">
         <v>120.3</v>
       </c>
       <c r="X23" s="3" t="n">
@@ -2494,8 +2494,8 @@
       <c r="Q24" s="8" t="n">
         <v>31.1</v>
       </c>
-      <c r="R24" s="9" t="n">
-        <v>23.8</v>
+      <c r="R24" s="8" t="n">
+        <v>25.6</v>
       </c>
       <c r="S24" s="8" t="n">
         <v>29.4</v>
@@ -2509,17 +2509,17 @@
       <c r="V24" s="8" t="n">
         <v>26.9</v>
       </c>
-      <c r="W24" s="9" t="n">
+      <c r="W24" s="8" t="n">
         <v>24.1</v>
       </c>
       <c r="X24" s="8" t="n">
-        <v>30</v>
+        <v>28.1</v>
       </c>
       <c r="Y24" s="8" t="n">
-        <v>84.7</v>
+        <v>79.2</v>
       </c>
       <c r="Z24" s="8" t="n">
-        <v>5.4</v>
+        <v>7.4</v>
       </c>
       <c r="AA24" s="3" t="inlineStr">
         <is>
@@ -2564,8 +2564,8 @@
       <c r="L25" s="8" t="n">
         <v>22.4</v>
       </c>
-      <c r="M25" s="10" t="n">
-        <v>98.09999999999999</v>
+      <c r="M25" s="8" t="n">
+        <v>21.9</v>
       </c>
       <c r="N25" s="3" t="n">
         <v>26.4</v>
@@ -2580,7 +2580,7 @@
         <v>26.2</v>
       </c>
       <c r="R25" s="8" t="n">
-        <v>23.4</v>
+        <v>24.1</v>
       </c>
       <c r="S25" s="8" t="n">
         <v>28.7</v>
@@ -2595,7 +2595,7 @@
         <v>24.4</v>
       </c>
       <c r="W25" s="8" t="n">
-        <v>22.2</v>
+        <v>22.8</v>
       </c>
       <c r="X25" s="8" t="n">
         <v>26.8</v>
@@ -2668,19 +2668,19 @@
         <v>23.3</v>
       </c>
       <c r="S26" s="8" t="n">
-        <v>28.6</v>
+        <v>27.9</v>
       </c>
       <c r="T26" s="8" t="n">
-        <v>94.2</v>
+        <v>91.90000000000001</v>
       </c>
       <c r="U26" s="8" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="V26" s="8" t="n">
         <v>23.8</v>
       </c>
       <c r="W26" s="8" t="n">
-        <v>22.4</v>
+        <v>22.8</v>
       </c>
       <c r="X26" s="8" t="n">
         <v>27.1</v>
@@ -2753,19 +2753,19 @@
         <v>24.9</v>
       </c>
       <c r="S27" s="8" t="n">
-        <v>31.5</v>
+        <v>28.8</v>
       </c>
       <c r="T27" s="8" t="n">
-        <v>79.5</v>
+        <v>72.7</v>
       </c>
       <c r="U27" s="8" t="n">
-        <v>8.1</v>
+        <v>10.8</v>
       </c>
       <c r="V27" s="8" t="n">
         <v>26.9</v>
       </c>
       <c r="W27" s="8" t="n">
-        <v>23.5</v>
+        <v>24.4</v>
       </c>
       <c r="X27" s="8" t="n">
         <v>29</v>
@@ -2835,7 +2835,7 @@
         <v>31.2</v>
       </c>
       <c r="R28" s="8" t="n">
-        <v>22.5</v>
+        <v>24.8</v>
       </c>
       <c r="S28" s="8" t="n">
         <v>27.2</v>
@@ -2850,7 +2850,7 @@
         <v>28.6</v>
       </c>
       <c r="W28" s="8" t="n">
-        <v>23.2</v>
+        <v>24.6</v>
       </c>
       <c r="X28" s="8" t="n">
         <v>28.4</v>
@@ -2904,23 +2904,23 @@
       <c r="L29" s="8" t="n">
         <v>21.1</v>
       </c>
-      <c r="M29" s="3" t="n">
+      <c r="M29" s="8" t="n">
         <v>20.6</v>
       </c>
-      <c r="N29" s="3" t="n">
+      <c r="N29" s="8" t="n">
         <v>23.9</v>
       </c>
-      <c r="O29" s="3" t="n">
-        <v>95.3</v>
-      </c>
-      <c r="P29" s="3" t="n">
+      <c r="O29" s="8" t="n">
+        <v>95.59999999999999</v>
+      </c>
+      <c r="P29" s="8" t="n">
         <v>1.1</v>
       </c>
       <c r="Q29" s="8" t="n">
         <v>25.3</v>
       </c>
       <c r="R29" s="8" t="n">
-        <v>22.9</v>
+        <v>23.6</v>
       </c>
       <c r="S29" s="8" t="n">
         <v>28</v>
@@ -2938,13 +2938,13 @@
         <v>21.3</v>
       </c>
       <c r="X29" s="8" t="n">
-        <v>25.3</v>
+        <v>24.6</v>
       </c>
       <c r="Y29" s="8" t="n">
-        <v>93.5</v>
+        <v>90.7</v>
       </c>
       <c r="Z29" s="8" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="AA29" s="3" t="inlineStr">
         <is>
@@ -2989,8 +2989,8 @@
       <c r="L30" s="8" t="n">
         <v>106.5</v>
       </c>
-      <c r="M30" s="9" t="n">
-        <v>105.2</v>
+      <c r="M30" s="8" t="n">
+        <v>105</v>
       </c>
       <c r="N30" s="3" t="n">
         <v>123.9</v>
@@ -3004,7 +3004,7 @@
       <c r="Q30" s="8" t="n">
         <v>135.8</v>
       </c>
-      <c r="R30" s="9" t="n">
+      <c r="R30" s="8" t="n">
         <v>120.7</v>
       </c>
       <c r="S30" s="3" t="n">
@@ -3019,7 +3019,7 @@
       <c r="V30" s="8" t="n">
         <v>126.1</v>
       </c>
-      <c r="W30" s="9" t="n">
+      <c r="W30" s="8" t="n">
         <v>115.9</v>
       </c>
       <c r="X30" s="3" t="n">
@@ -3072,14 +3072,14 @@
       <c r="L31" s="8" t="n">
         <v>21.3</v>
       </c>
-      <c r="M31" s="9" t="n">
+      <c r="M31" s="8" t="n">
         <v>21</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>24.8</v>
+        <v>24.7</v>
       </c>
       <c r="O31" s="8" t="n">
-        <v>97.5</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="P31" s="8" t="n">
         <v>0.6</v>
@@ -3087,32 +3087,32 @@
       <c r="Q31" s="8" t="n">
         <v>27.2</v>
       </c>
-      <c r="R31" s="9" t="n">
+      <c r="R31" s="8" t="n">
         <v>24.1</v>
       </c>
       <c r="S31" s="8" t="n">
-        <v>30</v>
+        <v>27.9</v>
       </c>
       <c r="T31" s="8" t="n">
-        <v>83.2</v>
+        <v>77.3</v>
       </c>
       <c r="U31" s="8" t="n">
-        <v>6.1</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="V31" s="8" t="n">
         <v>25.2</v>
       </c>
-      <c r="W31" s="9" t="n">
+      <c r="W31" s="8" t="n">
         <v>23.2</v>
       </c>
       <c r="X31" s="8" t="n">
-        <v>28.4</v>
+        <v>27.1</v>
       </c>
       <c r="Y31" s="8" t="n">
-        <v>88.7</v>
+        <v>84.40000000000001</v>
       </c>
       <c r="Z31" s="8" t="n">
-        <v>3.6</v>
+        <v>5</v>
       </c>
       <c r="AA31" s="3" t="inlineStr">
         <is>
@@ -3173,7 +3173,7 @@
         <v>31.1</v>
       </c>
       <c r="R32" s="8" t="n">
-        <v>22.7</v>
+        <v>24.9</v>
       </c>
       <c r="S32" s="8" t="n">
         <v>27.5</v>
@@ -3188,7 +3188,7 @@
         <v>27.4</v>
       </c>
       <c r="W32" s="8" t="n">
-        <v>22.5</v>
+        <v>23.8</v>
       </c>
       <c r="X32" s="8" t="n">
         <v>27.2</v>
@@ -3246,10 +3246,10 @@
         <v>21.4</v>
       </c>
       <c r="N33" s="8" t="n">
-        <v>25.5</v>
+        <v>25.4</v>
       </c>
       <c r="O33" s="8" t="n">
-        <v>99.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="P33" s="8" t="n">
         <v>0.2</v>
@@ -3258,7 +3258,7 @@
         <v>28.9</v>
       </c>
       <c r="R33" s="8" t="n">
-        <v>23.1</v>
+        <v>24.6</v>
       </c>
       <c r="S33" s="8" t="n">
         <v>28.2</v>
@@ -3276,13 +3276,13 @@
         <v>23.8</v>
       </c>
       <c r="X33" s="8" t="n">
-        <v>29.5</v>
+        <v>28.2</v>
       </c>
       <c r="Y33" s="8" t="n">
-        <v>89.8</v>
+        <v>86</v>
       </c>
       <c r="Z33" s="8" t="n">
-        <v>3.4</v>
+        <v>4.6</v>
       </c>
       <c r="AA33" s="3" t="inlineStr">
         <is>
@@ -3334,7 +3334,7 @@
         <v>25.9</v>
       </c>
       <c r="O34" s="8" t="n">
-        <v>99.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="P34" s="8" t="n">
         <v>0.2</v>
@@ -3343,7 +3343,7 @@
         <v>30.5</v>
       </c>
       <c r="R34" s="8" t="n">
-        <v>24.2</v>
+        <v>25.8</v>
       </c>
       <c r="S34" s="8" t="n">
         <v>30.2</v>
@@ -3358,7 +3358,7 @@
         <v>27.3</v>
       </c>
       <c r="W34" s="8" t="n">
-        <v>23.9</v>
+        <v>24.8</v>
       </c>
       <c r="X34" s="8" t="n">
         <v>29.7</v>
@@ -3428,7 +3428,7 @@
         <v>31.1</v>
       </c>
       <c r="R35" s="8" t="n">
-        <v>22.7</v>
+        <v>24.9</v>
       </c>
       <c r="S35" s="8" t="n">
         <v>27.5</v>
@@ -3443,7 +3443,7 @@
         <v>27.8</v>
       </c>
       <c r="W35" s="8" t="n">
-        <v>23.5</v>
+        <v>24.6</v>
       </c>
       <c r="X35" s="8" t="n">
         <v>28.9</v>
@@ -3501,19 +3501,19 @@
         <v>20.7</v>
       </c>
       <c r="N36" s="8" t="n">
-        <v>24.4</v>
+        <v>24.2</v>
       </c>
       <c r="O36" s="8" t="n">
-        <v>98.2</v>
+        <v>97.3</v>
       </c>
       <c r="P36" s="8" t="n">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="Q36" s="8" t="n">
         <v>32.1</v>
       </c>
       <c r="R36" s="8" t="n">
-        <v>23.9</v>
+        <v>26</v>
       </c>
       <c r="S36" s="8" t="n">
         <v>29.7</v>
@@ -3528,7 +3528,7 @@
         <v>28.7</v>
       </c>
       <c r="W36" s="8" t="n">
-        <v>23.1</v>
+        <v>24.6</v>
       </c>
       <c r="X36" s="8" t="n">
         <v>28.3</v>
@@ -3597,7 +3597,7 @@
       <c r="Q37" s="8" t="n">
         <v>153.7</v>
       </c>
-      <c r="R37" s="9" t="n">
+      <c r="R37" s="8" t="n">
         <v>126.2</v>
       </c>
       <c r="S37" s="3" t="n">
@@ -3612,7 +3612,7 @@
       <c r="V37" s="8" t="n">
         <v>136.8</v>
       </c>
-      <c r="W37" s="9" t="n">
+      <c r="W37" s="8" t="n">
         <v>121.6</v>
       </c>
       <c r="X37" s="3" t="n">
@@ -3669,19 +3669,19 @@
         <v>21</v>
       </c>
       <c r="N38" s="8" t="n">
-        <v>24.9</v>
+        <v>24.7</v>
       </c>
       <c r="O38" s="8" t="n">
-        <v>98.8</v>
+        <v>98.2</v>
       </c>
       <c r="P38" s="8" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="Q38" s="8" t="n">
         <v>30.7</v>
       </c>
-      <c r="R38" s="9" t="n">
-        <v>23.3</v>
+      <c r="R38" s="8" t="n">
+        <v>25.2</v>
       </c>
       <c r="S38" s="8" t="n">
         <v>28.6</v>
@@ -3695,8 +3695,8 @@
       <c r="V38" s="8" t="n">
         <v>27.4</v>
       </c>
-      <c r="W38" s="9" t="n">
-        <v>23.2</v>
+      <c r="W38" s="8" t="n">
+        <v>24.3</v>
       </c>
       <c r="X38" s="8" t="n">
         <v>28.5</v>
@@ -3766,7 +3766,7 @@
         <v>31.9</v>
       </c>
       <c r="R39" s="8" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="S39" s="8" t="n">
         <v>29.8</v>
@@ -3784,13 +3784,13 @@
         <v>23.2</v>
       </c>
       <c r="X39" s="8" t="n">
-        <v>28.4</v>
+        <v>27.4</v>
       </c>
       <c r="Y39" s="8" t="n">
-        <v>91.40000000000001</v>
+        <v>88.09999999999999</v>
       </c>
       <c r="Z39" s="8" t="n">
-        <v>2.7</v>
+        <v>3.7</v>
       </c>
       <c r="AA39" s="3" t="inlineStr">
         <is>
@@ -3851,7 +3851,7 @@
         <v>32.8</v>
       </c>
       <c r="R40" s="8" t="n">
-        <v>23.7</v>
+        <v>26</v>
       </c>
       <c r="S40" s="8" t="n">
         <v>29.3</v>
@@ -3869,13 +3869,13 @@
         <v>23.8</v>
       </c>
       <c r="X40" s="8" t="n">
-        <v>29.5</v>
+        <v>26.7</v>
       </c>
       <c r="Y40" s="8" t="n">
-        <v>78.90000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="Z40" s="8" t="n">
-        <v>7.9</v>
+        <v>10.6</v>
       </c>
       <c r="AA40" s="3" t="inlineStr">
         <is>
@@ -3939,19 +3939,19 @@
         <v>21.4</v>
       </c>
       <c r="S41" s="8" t="n">
-        <v>25.5</v>
+        <v>24.9</v>
       </c>
       <c r="T41" s="8" t="n">
-        <v>94.59999999999999</v>
+        <v>92.40000000000001</v>
       </c>
       <c r="U41" s="8" t="n">
-        <v>1.4</v>
+        <v>2.1</v>
       </c>
       <c r="V41" s="8" t="n">
         <v>24.6</v>
       </c>
       <c r="W41" s="8" t="n">
-        <v>22.9</v>
+        <v>23.4</v>
       </c>
       <c r="X41" s="8" t="n">
         <v>28</v>
@@ -4009,10 +4009,10 @@
         <v>21.8</v>
       </c>
       <c r="N42" s="8" t="n">
-        <v>26.1</v>
+        <v>26</v>
       </c>
       <c r="O42" s="8" t="n">
-        <v>99.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="P42" s="8" t="n">
         <v>0.2</v>
@@ -4039,13 +4039,13 @@
         <v>23.5</v>
       </c>
       <c r="X42" s="8" t="n">
-        <v>28.9</v>
+        <v>28.1</v>
       </c>
       <c r="Y42" s="8" t="n">
-        <v>93</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="Z42" s="8" t="n">
-        <v>2.2</v>
+        <v>3</v>
       </c>
       <c r="AA42" s="3" t="inlineStr">
         <is>
@@ -4097,7 +4097,7 @@
         <v>25.6</v>
       </c>
       <c r="O43" s="8" t="n">
-        <v>99.40000000000001</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="P43" s="8" t="n">
         <v>0.2</v>
@@ -4106,7 +4106,7 @@
         <v>29.1</v>
       </c>
       <c r="R43" s="8" t="n">
-        <v>24.3</v>
+        <v>25.5</v>
       </c>
       <c r="S43" s="8" t="n">
         <v>30.4</v>
@@ -4124,13 +4124,13 @@
         <v>24.7</v>
       </c>
       <c r="X43" s="8" t="n">
-        <v>31.1</v>
+        <v>29</v>
       </c>
       <c r="Y43" s="8" t="n">
-        <v>83.3</v>
+        <v>77.5</v>
       </c>
       <c r="Z43" s="8" t="n">
-        <v>6.3</v>
+        <v>8.4</v>
       </c>
       <c r="AA43" s="3" t="inlineStr">
         <is>
@@ -4191,7 +4191,7 @@
         <v>32.6</v>
       </c>
       <c r="R44" s="8" t="n">
-        <v>24.3</v>
+        <v>26.4</v>
       </c>
       <c r="S44" s="8" t="n">
         <v>30.4</v>
@@ -4206,7 +4206,7 @@
         <v>28.5</v>
       </c>
       <c r="W44" s="8" t="n">
-        <v>25.6</v>
+        <v>26.3</v>
       </c>
       <c r="X44" s="8" t="n">
         <v>32.8</v>
@@ -4275,7 +4275,7 @@
       <c r="Q45" s="8" t="n">
         <v>172.8</v>
       </c>
-      <c r="R45" s="9" t="n">
+      <c r="R45" s="8" t="n">
         <v>149.1</v>
       </c>
       <c r="S45" s="3" t="n">
@@ -4290,7 +4290,7 @@
       <c r="V45" s="8" t="n">
         <v>158.1</v>
       </c>
-      <c r="W45" s="9" t="n">
+      <c r="W45" s="8" t="n">
         <v>144.9</v>
       </c>
       <c r="X45" s="3" t="n">
@@ -4360,32 +4360,32 @@
       <c r="Q46" s="8" t="n">
         <v>28.8</v>
       </c>
-      <c r="R46" s="9" t="n">
+      <c r="R46" s="8" t="n">
         <v>24.8</v>
       </c>
       <c r="S46" s="8" t="n">
-        <v>31.3</v>
+        <v>28.5</v>
       </c>
       <c r="T46" s="8" t="n">
-        <v>79</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="U46" s="8" t="n">
-        <v>8.300000000000001</v>
+        <v>11.1</v>
       </c>
       <c r="V46" s="8" t="n">
         <v>26.3</v>
       </c>
-      <c r="W46" s="9" t="n">
+      <c r="W46" s="8" t="n">
         <v>24.1</v>
       </c>
       <c r="X46" s="8" t="n">
-        <v>30</v>
+        <v>28.5</v>
       </c>
       <c r="Y46" s="8" t="n">
-        <v>87.7</v>
+        <v>83.3</v>
       </c>
       <c r="Z46" s="8" t="n">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
       <c r="AA46" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Results from updated MeteoSaver v1.0 to also QA/QC confirm precipitation values in addition to temperature values
</commit_message>
<xml_diff>
--- a/results/02_post_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_post_QA_QC.xlsx
+++ b/results/02_post_QA_QC_transcribed_hydroclimate_data/203/203_196905_SF.JPG_post_QA_QC.xlsx
@@ -26,7 +26,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +55,18 @@
       <patternFill patternType="solid">
         <fgColor rgb="0075696F"/>
         <bgColor rgb="0075696F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFC0CB"/>
+        <bgColor rgb="00FFC0CB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -125,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment textRotation="90"/>
@@ -155,6 +167,12 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -162,6 +180,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -798,7 +819,7 @@
       <c r="J4" s="3" t="n">
         <v>9.9</v>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="K4" s="10" t="n">
         <v>0</v>
       </c>
       <c r="L4" s="3" t="n">
@@ -883,7 +904,7 @@
       <c r="J5" s="3" t="n">
         <v>5.5</v>
       </c>
-      <c r="K5" s="3" t="n">
+      <c r="K5" s="10" t="n">
         <v>0</v>
       </c>
       <c r="L5" s="3" t="n">
@@ -968,7 +989,7 @@
       <c r="J6" s="3" t="n">
         <v>7.2</v>
       </c>
-      <c r="K6" s="3" t="n">
+      <c r="K6" s="10" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="3" t="n">
@@ -1053,7 +1074,7 @@
       <c r="J7" s="3" t="n">
         <v>1.9</v>
       </c>
-      <c r="K7" s="3" t="n">
+      <c r="K7" s="10" t="n">
         <v>0</v>
       </c>
       <c r="L7" s="3" t="n">
@@ -1138,7 +1159,7 @@
       <c r="J8" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="K8" s="3" t="n">
+      <c r="K8" s="10" t="n">
         <v>30.9</v>
       </c>
       <c r="L8" s="3" t="n">
@@ -1223,7 +1244,7 @@
       <c r="J9" s="3" t="n">
         <v>27.5</v>
       </c>
-      <c r="K9" s="3" t="n">
+      <c r="K9" s="10" t="n">
         <v>30.9</v>
       </c>
       <c r="L9" s="3" t="n">
@@ -1814,7 +1835,7 @@
       <c r="J16" s="3" t="n">
         <v>19.4</v>
       </c>
-      <c r="K16" s="3" t="n"/>
+      <c r="K16" s="13" t="n"/>
       <c r="L16" s="3" t="n"/>
       <c r="M16" s="3" t="n">
         <v>109.5</v>
@@ -1978,7 +1999,7 @@
       <c r="J18" s="3" t="n">
         <v>14.3</v>
       </c>
-      <c r="K18" s="3" t="n"/>
+      <c r="K18" s="14" t="n"/>
       <c r="L18" s="3" t="n">
         <v>22.1</v>
       </c>
@@ -2401,7 +2422,7 @@
       <c r="J23" s="3" t="n">
         <v>19.3</v>
       </c>
-      <c r="K23" s="3" t="n">
+      <c r="K23" s="18" t="n">
         <v>7.7</v>
       </c>
       <c r="L23" s="3" t="n">
@@ -2996,7 +3017,7 @@
       <c r="J30" s="3" t="n">
         <v>111</v>
       </c>
-      <c r="K30" s="3" t="n">
+      <c r="K30" s="18" t="n">
         <v>38.8</v>
       </c>
       <c r="L30" s="3" t="n">
@@ -3591,7 +3612,7 @@
       <c r="J37" s="3" t="n">
         <v>0.4</v>
       </c>
-      <c r="K37" s="3" t="n">
+      <c r="K37" s="18" t="n">
         <v>35.6</v>
       </c>
       <c r="L37" s="3" t="n">
@@ -4271,7 +4292,7 @@
       <c r="J45" s="3" t="n">
         <v>18.8</v>
       </c>
-      <c r="K45" s="3" t="n">
+      <c r="K45" s="18" t="n">
         <v>0</v>
       </c>
       <c r="L45" s="3" t="n">

</xml_diff>